<commit_message>
Fixed comments from copilot
</commit_message>
<xml_diff>
--- a/api_pca_results.xlsx
+++ b/api_pca_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance Explained" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loadings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded APIs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Variance Explained" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Loadings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Scores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Excluded APIs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,13 +448,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6909094175621651</v>
+        <v>0.7396822596646899</v>
       </c>
       <c r="C2" t="n">
-        <v>69.09094175621651</v>
+        <v>73.96822596646899</v>
       </c>
       <c r="D2" t="n">
-        <v>69.09094175621651</v>
+        <v>73.96822596646899</v>
       </c>
     </row>
     <row r="3">
@@ -464,13 +464,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1322712315496568</v>
+        <v>0.1184354314738571</v>
       </c>
       <c r="C3" t="n">
-        <v>13.22712315496568</v>
+        <v>11.84354314738571</v>
       </c>
       <c r="D3" t="n">
-        <v>82.31806491118219</v>
+        <v>85.81176911385471</v>
       </c>
     </row>
     <row r="4">
@@ -480,13 +480,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.09527576077031397</v>
+        <v>0.07885988345682321</v>
       </c>
       <c r="C4" t="n">
-        <v>9.527576077031396</v>
+        <v>7.885988345682321</v>
       </c>
       <c r="D4" t="n">
-        <v>91.84564098821359</v>
+        <v>93.69775745953703</v>
       </c>
     </row>
     <row r="5">
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04393982425387265</v>
+        <v>0.04501137305239598</v>
       </c>
       <c r="C5" t="n">
-        <v>4.393982425387264</v>
+        <v>4.501137305239598</v>
       </c>
       <c r="D5" t="n">
-        <v>96.23962341360085</v>
+        <v>98.19889476477664</v>
       </c>
     </row>
     <row r="6">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.03014459500523198</v>
+        <v>0.01325358807765344</v>
       </c>
       <c r="C6" t="n">
-        <v>3.014459500523198</v>
+        <v>1.325358807765344</v>
       </c>
       <c r="D6" t="n">
-        <v>99.25408291412406</v>
+        <v>99.52425357254198</v>
       </c>
     </row>
     <row r="7">
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.003804775983399328</v>
+        <v>0.00282747772541384</v>
       </c>
       <c r="C7" t="n">
-        <v>0.3804775983399328</v>
+        <v>0.282747772541384</v>
       </c>
       <c r="D7" t="n">
-        <v>99.63456051246399</v>
+        <v>99.80700134508336</v>
       </c>
     </row>
     <row r="8">
@@ -544,13 +544,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001757509553373926</v>
+        <v>0.0009842637891835004</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1757509553373926</v>
+        <v>0.09842637891835004</v>
       </c>
       <c r="D8" t="n">
-        <v>99.81031146780138</v>
+        <v>99.90542772400171</v>
       </c>
     </row>
     <row r="9">
@@ -560,13 +560,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001338457552070829</v>
+        <v>0.0006920096145600679</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1338457552070829</v>
+        <v>0.06920096145600679</v>
       </c>
       <c r="D9" t="n">
-        <v>99.94415722300846</v>
+        <v>99.97462868545772</v>
       </c>
     </row>
     <row r="10">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0004828044877045719</v>
+        <v>0.0001967862565253606</v>
       </c>
       <c r="C10" t="n">
-        <v>0.04828044877045719</v>
+        <v>0.01967862565253605</v>
       </c>
       <c r="D10" t="n">
-        <v>99.99243767177892</v>
+        <v>99.99430731111025</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.633433764934852e-05</v>
+        <v>4.039334361622885e-05</v>
       </c>
       <c r="C11" t="n">
-        <v>0.006633433764934853</v>
+        <v>0.004039334361622885</v>
       </c>
       <c r="D11" t="n">
-        <v>99.99907110554386</v>
+        <v>99.99834664547187</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.288944561527606e-06</v>
+        <v>1.653354528114542e-05</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0009288944561527606</v>
+        <v>0.001653354528114542</v>
       </c>
       <c r="D12" t="n">
-        <v>100</v>
+        <v>99.99999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -695,37 +695,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.359930078057726</v>
+        <v>0.3480441041852776</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05214642167688733</v>
+        <v>0.04840257616094605</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0588769658186173</v>
+        <v>0.0395850795322399</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06697435293573306</v>
+        <v>-0.07044592927863616</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.1050459294534209</v>
+        <v>0.1227340622519716</v>
       </c>
       <c r="G2" t="n">
-        <v>0.005599059603605696</v>
+        <v>0.3489385360214914</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0499956063109356</v>
+        <v>-0.08294085362001047</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3120710124803681</v>
+        <v>-0.4144835056110443</v>
       </c>
       <c r="J2" t="n">
-        <v>0.07753844454754273</v>
+        <v>-0.1571621003056827</v>
       </c>
       <c r="K2" t="n">
-        <v>0.812549639255092</v>
+        <v>-0.1109574816719508</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.2873604490530284</v>
+        <v>0.7193635260404461</v>
       </c>
     </row>
     <row r="3">
@@ -735,37 +735,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.1933713291104824</v>
+        <v>-0.2717844848700969</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5597953669010864</v>
+        <v>0.4600596601471946</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1667552123703212</v>
+        <v>-0.1555368520902943</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5742503176944909</v>
+        <v>0.223475675715559</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.4558332860619624</v>
+        <v>0.720643180761425</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.2161672402649482</v>
+        <v>0.1723064116028518</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1442056330483297</v>
+        <v>0.278423950860016</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.05992937101361172</v>
+        <v>0.08087387598281544</v>
       </c>
       <c r="J3" t="n">
-        <v>0.06591124085325513</v>
+        <v>-0.0003515313889551203</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.07695517610802288</v>
+        <v>0.08374251800218749</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.05000502664562545</v>
+        <v>0.01599081962926729</v>
       </c>
     </row>
     <row r="4">
@@ -775,37 +775,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.332943126177018</v>
+        <v>0.3304195706146875</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.1365936234304379</v>
+        <v>-0.1619310960143837</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2399720262964883</v>
+        <v>0.1621051707555164</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1002126826866405</v>
+        <v>0.1430348306248074</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.3696067415273857</v>
+        <v>0.4918425292955053</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6162578497296092</v>
+        <v>-0.4197663500681541</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1478352804554556</v>
+        <v>-0.5448147945544466</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.4857712284037868</v>
+        <v>0.2768259899287904</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.1268888604063896</v>
+        <v>-0.1478079368384611</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.04491476221485941</v>
+        <v>0.04687917767652454</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.1026252678698205</v>
+        <v>0.04744136918318019</v>
       </c>
     </row>
     <row r="5">
@@ -815,37 +815,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3582809265001394</v>
+        <v>0.3436447736645724</v>
       </c>
       <c r="C5" t="n">
-        <v>0.06404951191994596</v>
+        <v>0.1092177379593841</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.02597646299276469</v>
+        <v>-0.01671977112053451</v>
       </c>
       <c r="E5" t="n">
-        <v>0.006756689216057959</v>
+        <v>-0.1250756199421833</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.04352534199109306</v>
+        <v>-0.09715381142050872</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.506675539855917</v>
+        <v>0.5801949996531719</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.4714647353368164</v>
+        <v>-0.03806377030439162</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.07144224510959211</v>
+        <v>0.7014635639584008</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.6101021284345518</v>
+        <v>-0.05587379391002843</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.07031324491197945</v>
+        <v>-0.07671459258153267</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.06038128504412387</v>
+        <v>-0.07405539392833699</v>
       </c>
     </row>
     <row r="6">
@@ -855,37 +855,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3534531749094307</v>
+        <v>0.3463977141952448</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.1471900950773364</v>
+        <v>-0.09687788400027632</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.01756042417979313</v>
+        <v>0.02498892564205073</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.05286349757737771</v>
+        <v>-0.04766242489352817</v>
       </c>
       <c r="F6" t="n">
-        <v>0.03901519430006663</v>
+        <v>0.05371991268105927</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.2828305394829376</v>
+        <v>-0.3480743404589615</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7935235909356777</v>
+        <v>0.6877572692733405</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.287815657923225</v>
+        <v>0.1038228181389322</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.1253594643912896</v>
+        <v>-0.4093847889325154</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.118424991998029</v>
+        <v>-0.3037746705301073</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.1628824587675511</v>
+        <v>-0.00462338257495204</v>
       </c>
     </row>
     <row r="7">
@@ -895,37 +895,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3597837649501694</v>
+        <v>0.3483766950177057</v>
       </c>
       <c r="C7" t="n">
-        <v>0.05908999943890125</v>
+        <v>0.04596915079947084</v>
       </c>
       <c r="D7" t="n">
-        <v>0.04989851029720357</v>
+        <v>0.03698802635088281</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06977912788737317</v>
+        <v>-0.04830070664152148</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1126318125535505</v>
+        <v>0.1439002603103246</v>
       </c>
       <c r="G7" t="n">
-        <v>0.09206032841784505</v>
+        <v>0.2731614965110287</v>
       </c>
       <c r="H7" t="n">
-        <v>0.154910490185699</v>
+        <v>-0.08886311896821164</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2653029908652605</v>
+        <v>-0.4729655601714178</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.08944013202539411</v>
+        <v>-0.2963297862608043</v>
       </c>
       <c r="K7" t="n">
-        <v>0.01278412001875755</v>
+        <v>0.1522207217869724</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8579033099863236</v>
+        <v>-0.6594841845765869</v>
       </c>
     </row>
     <row r="8">
@@ -935,37 +935,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3556683618131856</v>
+        <v>0.348590672645173</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.08963190058747653</v>
+        <v>-0.06761960552236101</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1221105868115283</v>
+        <v>0.05751176825984187</v>
       </c>
       <c r="E8" t="n">
-        <v>0.004797335575314143</v>
+        <v>-0.03752206718068614</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0197806450287403</v>
+        <v>-0.003404444973988396</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.3670960483671938</v>
+        <v>-0.07865818230381347</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.2754346044268136</v>
+        <v>0.3108627720143484</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.2759735460148386</v>
+        <v>0.04223580640118429</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7402336576085935</v>
+        <v>0.319779170939097</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.06660443967018598</v>
+        <v>0.8046427127606141</v>
       </c>
       <c r="L8" t="n">
-        <v>0.10475546602171</v>
+        <v>0.1219417207477423</v>
       </c>
     </row>
     <row r="9">
@@ -975,37 +975,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.3591676796051365</v>
+        <v>0.3468107306911331</v>
       </c>
       <c r="C9" t="n">
-        <v>0.004781850942726346</v>
+        <v>0.06927662248080196</v>
       </c>
       <c r="D9" t="n">
-        <v>0.09837778228534266</v>
+        <v>-0.01755600620588045</v>
       </c>
       <c r="E9" t="n">
-        <v>0.06412917098272033</v>
+        <v>-0.1275281437178474</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.03653375962038505</v>
+        <v>0.1881477230962233</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1507730852879752</v>
+        <v>-0.06661008130287661</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.007660571439159443</v>
+        <v>0.05113272283554106</v>
       </c>
       <c r="I9" t="n">
-        <v>0.623360046003389</v>
+        <v>-0.1243647453691872</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1169902865380097</v>
+        <v>0.759887735282643</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.5528145574728895</v>
+        <v>-0.44694779502802</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.3538228949131769</v>
+        <v>-0.1524536331968943</v>
       </c>
     </row>
     <row r="10">
@@ -1015,37 +1015,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1416430339851202</v>
+        <v>0.2574287906374266</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4611261119434677</v>
+        <v>0.1679571146662453</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.5959407418981854</v>
+        <v>-0.1719811428985963</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.5069328964102605</v>
+        <v>0.8818659623884528</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.3526958699109341</v>
+        <v>-0.3022065344352616</v>
       </c>
       <c r="G10" t="n">
-        <v>0.08880941307548043</v>
+        <v>-0.01121982199923165</v>
       </c>
       <c r="H10" t="n">
-        <v>0.002659851477508381</v>
+        <v>-0.01328354625147483</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.06974272286947433</v>
+        <v>-0.03539646903607532</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1184332832315036</v>
+        <v>0.04586766351738255</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.05130965498940506</v>
+        <v>-0.05704346125158385</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.03690388207272022</v>
+        <v>-0.003728369820071527</v>
       </c>
     </row>
     <row r="11">
@@ -1055,77 +1055,77 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.06050523961135032</v>
+        <v>0.01156641681075643</v>
       </c>
       <c r="C11" t="n">
-        <v>0.5716261712982318</v>
+        <v>0.6381336580720642</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5967438444552544</v>
+        <v>0.7294267861505931</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.4034066917694585</v>
+        <v>-0.04758114842870974</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3662928387673864</v>
+        <v>-0.185448902484309</v>
       </c>
       <c r="G11" t="n">
-        <v>0.07839410859428647</v>
+        <v>-0.1512893948276761</v>
       </c>
       <c r="H11" t="n">
-        <v>0.03601516013173722</v>
+        <v>-0.02287883588383523</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.08456528991558852</v>
+        <v>0.000251234724914865</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.04273112858542336</v>
+        <v>-0.02211404971593781</v>
       </c>
       <c r="K11" t="n">
-        <v>0.003496736918279016</v>
+        <v>-0.004261008262157466</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.01182475687855738</v>
+        <v>0.003712457602717819</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>number_of_rings_calc</t>
+          <t>number_of_rings</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2454444484706371</v>
+        <v>0.1678555032098235</v>
       </c>
       <c r="C12" t="n">
-        <v>0.2975612093506695</v>
+        <v>0.5399609235365636</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.4145224420624015</v>
+        <v>-0.6167935998218748</v>
       </c>
       <c r="E12" t="n">
-        <v>0.473440189004416</v>
+        <v>-0.3267500277830358</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6067774293475854</v>
+        <v>-0.1718646691793672</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2382300075690835</v>
+        <v>-0.3260537451065727</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.04082751954775142</v>
+        <v>-0.1909766476838945</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.1672257824476509</v>
+        <v>0.0002333491717852951</v>
       </c>
       <c r="J12" t="n">
-        <v>0.01088983349360525</v>
+        <v>-0.1124396452737646</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.002605702479669583</v>
+        <v>0.0815984312712674</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.02346848457370656</v>
+        <v>0.0380155786551334</v>
       </c>
     </row>
   </sheetData>
@@ -1139,7 +1139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1211,37 +1211,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.52765389746596</v>
+        <v>0.4994196562552905</v>
       </c>
       <c r="C2" t="n">
-        <v>2.031726514526741</v>
+        <v>2.472678638941129</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8658148441359298</v>
+        <v>0.3682638423581847</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5970451913324593</v>
+        <v>-0.4841451139010026</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5919027079286111</v>
+        <v>0.3303438807789143</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.4942498589958755</v>
+        <v>0.1065663275750653</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.1902812019769515</v>
+        <v>0.1022095167285055</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.1224566242462999</v>
+        <v>0.1891933688824013</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1290047845027848</v>
+        <v>0.1127146836797746</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.005778603534669141</v>
+        <v>-0.03235178406878325</v>
       </c>
       <c r="L2" t="n">
-        <v>0.005440096284295626</v>
+        <v>0.0006366664350142242</v>
       </c>
     </row>
     <row r="3">
@@ -1251,37 +1251,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.204500033992767</v>
+        <v>2.518194283051294</v>
       </c>
       <c r="C3" t="n">
-        <v>-1.132573392470327</v>
+        <v>-0.7846411752384059</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.3610088706900949</v>
+        <v>0.01962216128453597</v>
       </c>
       <c r="E3" t="n">
-        <v>-1.07215018423866</v>
+        <v>0.08981860151928035</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.7606141193272649</v>
+        <v>-0.4004249035431454</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1423790614405324</v>
+        <v>0.1012289689359072</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.07376854512258753</v>
+        <v>0.1081782169677781</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.2329080434373564</v>
+        <v>-0.0800810654884255</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.006180217588686716</v>
+        <v>0.09776920707564295</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.04468288372526845</v>
+        <v>0.0523890689825259</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01446359138222788</v>
+        <v>-0.02490192027989758</v>
       </c>
     </row>
     <row r="4">
@@ -1291,73 +1291,77 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.077381291819992</v>
+        <v>-1.84364081844942</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.313147911240408</v>
+        <v>-1.296221089181179</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3029918685019233</v>
+        <v>0.5322411559964286</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.6077405630814668</v>
+        <v>0.01124748356239265</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05801130287541439</v>
+        <v>-0.2200723542953316</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06192249396377142</v>
+        <v>-0.09930281003495653</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1459841379055718</v>
+        <v>0.106160684629904</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02030970993917637</v>
+        <v>-0.09675655750282203</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1310985303288692</v>
+        <v>0.01005955453971012</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.003667679821591379</v>
+        <v>-0.01391325337486565</v>
       </c>
       <c r="L4" t="n">
-        <v>0.007038245614320882</v>
+        <v>0.0005222115222033951</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cathelicidin (LL37)</t>
+        </is>
+      </c>
       <c r="B5" t="n">
-        <v>0.1686770439500241</v>
+        <v>11.23039066909353</v>
       </c>
       <c r="C5" t="n">
-        <v>3.877964320618791</v>
+        <v>-1.422663573121028</v>
       </c>
       <c r="D5" t="n">
-        <v>1.711230350845324</v>
+        <v>0.6659723395951535</v>
       </c>
       <c r="E5" t="n">
-        <v>-1.324300106228617</v>
+        <v>1.317476102034821</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1383061572649822</v>
+        <v>0.4962108703658131</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1544996026428347</v>
+        <v>-0.2542860730991719</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1457440809774228</v>
+        <v>-0.03935772062311443</v>
       </c>
       <c r="I5" t="n">
-        <v>0.136807430427869</v>
+        <v>0.05289304574184379</v>
       </c>
       <c r="J5" t="n">
-        <v>0.02564563347111994</v>
+        <v>0.004977187612214575</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.007041789413938058</v>
+        <v>-0.007591791906127566</v>
       </c>
       <c r="L5" t="n">
-        <v>0.005776905626336868</v>
+        <v>0.002280224059648944</v>
       </c>
     </row>
     <row r="6">
@@ -1367,37 +1371,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.241083001389164</v>
+        <v>-0.3544797707292202</v>
       </c>
       <c r="C6" t="n">
-        <v>-1.01781586587233</v>
+        <v>3.370109261913631</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3235956199632501</v>
+        <v>2.518330746021151</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.3917013588531116</v>
+        <v>0.9202304622335878</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.08071644765175409</v>
+        <v>-0.2547031258630256</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1625684334671421</v>
+        <v>-0.04824045660832674</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1751987348683658</v>
+        <v>0.02520846413451666</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1175736321206431</v>
+        <v>-0.1379540081717562</v>
       </c>
       <c r="J6" t="n">
-        <v>0.04433163456634966</v>
+        <v>-0.03024812048719854</v>
       </c>
       <c r="K6" t="n">
-        <v>0.05506973265536707</v>
+        <v>0.009140420378840669</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.01284368817927977</v>
+        <v>-0.0004854918345328356</v>
       </c>
     </row>
     <row r="7">
@@ -1407,37 +1411,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.1417261280226247</v>
+        <v>-1.853105967891027</v>
       </c>
       <c r="C7" t="n">
-        <v>1.017702704560922</v>
+        <v>-1.261267475422086</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.147268836479328</v>
+        <v>0.5249731116318999</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.5099214816031322</v>
+        <v>-0.008198063287445425</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.360376365886462</v>
+        <v>-0.2728112856173099</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.08150379452755789</v>
+        <v>0.1000397417737514</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1344514496001193</v>
+        <v>-0.05890771896352544</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1071527858080859</v>
+        <v>0.04261231045161718</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0461397362480622</v>
+        <v>0.06910302467520685</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.006333457733748572</v>
+        <v>0.004870169613261754</v>
       </c>
       <c r="L7" t="n">
-        <v>0.005826526668282575</v>
+        <v>0.03630489053742018</v>
       </c>
     </row>
     <row r="8">
@@ -1447,37 +1451,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.411158396042518</v>
+        <v>-0.2984695197554383</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01180982744350941</v>
+        <v>0.03708503297232664</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.5358831297099353</v>
+        <v>-0.430342098334104</v>
       </c>
       <c r="E8" t="n">
-        <v>0.256063931940864</v>
+        <v>1.388665331647193</v>
       </c>
       <c r="F8" t="n">
-        <v>0.05893114199567174</v>
+        <v>-0.1250990702351577</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.1454239045762561</v>
+        <v>0.4767666924061776</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.03193366908668248</v>
+        <v>-0.02225510521777503</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.05058536289848176</v>
+        <v>0.04654889665497481</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.03604613951691361</v>
+        <v>-0.02119042365839661</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.05293229863413423</v>
+        <v>-0.04258423862270947</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.01178132322977382</v>
+        <v>-0.01235764574545984</v>
       </c>
     </row>
     <row r="9">
@@ -1487,73 +1491,77 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-1.634909272917</v>
+        <v>-0.5137953612039901</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.1375760285559779</v>
+        <v>-0.1157396809219698</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2323549278159164</v>
+        <v>-0.5345292425711552</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7383636207216366</v>
+        <v>-0.07820120817246806</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1862366811039766</v>
+        <v>-0.2793055195670694</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1188926703567983</v>
+        <v>-0.0314415688383424</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.05413578305887547</v>
+        <v>-0.06297643852929412</v>
       </c>
       <c r="I9" t="n">
-        <v>0.152952166971552</v>
+        <v>0.1044781732223136</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.06703499977998734</v>
+        <v>-0.02246166071738499</v>
       </c>
       <c r="K9" t="n">
-        <v>0.01832935125718557</v>
+        <v>0.01180378141762061</v>
       </c>
       <c r="L9" t="n">
-        <v>0.01193408467948657</v>
+        <v>-0.01550128915383261</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bortezomib</t>
+        </is>
+      </c>
       <c r="B10" t="n">
-        <v>0.05250486854365183</v>
+        <v>-1.230498008401778</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9772692262859021</v>
+        <v>-0.7368187691394492</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.952298389915547</v>
+        <v>0.1154506504990819</v>
       </c>
       <c r="E10" t="n">
-        <v>1.224096950457258</v>
+        <v>0.0003106754836107111</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1324102928891745</v>
+        <v>0.08011496636265077</v>
       </c>
       <c r="G10" t="n">
-        <v>0.6089366065331937</v>
+        <v>-0.03446608198497465</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1991450747103832</v>
+        <v>-0.05033907337489325</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1876837124996352</v>
+        <v>0.001727926765278782</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.01795090603639355</v>
+        <v>-0.05056704847719513</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.02693418048730904</v>
+        <v>-0.01314870591834223</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.0007686418922566304</v>
+        <v>-0.00802726255141864</v>
       </c>
     </row>
     <row r="11">
@@ -1563,37 +1571,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.9040831937852458</v>
+        <v>-1.641610848838819</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.1854590047256248</v>
+        <v>-0.2510166888682236</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.01199317107188016</v>
+        <v>-0.1885551822924716</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8695602232804758</v>
+        <v>-0.1411560352501725</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2665499522923722</v>
+        <v>0.5140902393882557</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1803658096651869</v>
+        <v>-0.00124645458198128</v>
       </c>
       <c r="H11" t="n">
-        <v>0.05634795798910824</v>
+        <v>0.02293024047162344</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.01699265935948073</v>
+        <v>-0.167952585268016</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.1297055213979117</v>
+        <v>0.08469848884430112</v>
       </c>
       <c r="K11" t="n">
-        <v>0.01160067821266483</v>
+        <v>0.006531560191316547</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02438081543726334</v>
+        <v>0.01012275231118172</v>
       </c>
     </row>
     <row r="12">
@@ -1603,73 +1611,73 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-1.709708840405548</v>
+        <v>-0.3930794990060364</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.4685183246473083</v>
+        <v>1.13865226421693</v>
       </c>
       <c r="D12" t="n">
-        <v>0.08661601543964403</v>
+        <v>-1.499934813156435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3873939233174259</v>
+        <v>-0.1038917388659296</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1547735186370727</v>
+        <v>0.3303547473777391</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.09404324250721927</v>
+        <v>-0.09484114557959519</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1267979128216733</v>
+        <v>-0.3248751749096153</v>
       </c>
       <c r="I12" t="n">
-        <v>0.05618060070139536</v>
+        <v>-0.1565109880937127</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.01003821532782837</v>
+        <v>0.04159834705758544</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.02390227041985087</v>
+        <v>-0.004352556418899105</v>
       </c>
       <c r="L12" t="n">
-        <v>0.002461326931445639</v>
+        <v>-0.01687876480850359</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>-2.073168711604271</v>
+        <v>-1.001180799576471</v>
       </c>
       <c r="C13" t="n">
-        <v>-1.095529323593049</v>
+        <v>0.004526488647274396</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1489999111583724</v>
+        <v>-0.5167039182971834</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.3982274261241155</v>
+        <v>-0.5092150947048052</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2252395318916355</v>
+        <v>0.2584201206651027</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00607418158620354</v>
+        <v>-0.01034181459199156</v>
       </c>
       <c r="H13" t="n">
-        <v>0.03002837405988893</v>
+        <v>0.03187105467832782</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1087001372557402</v>
+        <v>0.101157913146768</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.01814220141847677</v>
+        <v>-0.04677486169473474</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.02111899112080894</v>
+        <v>0.03141669801518642</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01154920334239618</v>
+        <v>-0.01265993121666253</v>
       </c>
     </row>
     <row r="14">
@@ -1679,73 +1687,73 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.821158792308981</v>
+        <v>-1.594132921442637</v>
       </c>
       <c r="C14" t="n">
-        <v>0.08450560816176959</v>
+        <v>-0.3476895016718284</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.3608845210158493</v>
+        <v>-0.1710043614234952</v>
       </c>
       <c r="E14" t="n">
-        <v>0.5727781942548477</v>
+        <v>-0.1995837348905727</v>
       </c>
       <c r="F14" t="n">
-        <v>0.06006543206819367</v>
+        <v>0.2901838727391026</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1283726602843552</v>
+        <v>-0.03302516042291687</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05790515840752997</v>
+        <v>0.1139580726504399</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.05782328398365907</v>
+        <v>0.01466665171961654</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.06036918447736052</v>
+        <v>0.02585817000003613</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.01843837355176594</v>
+        <v>-0.007679230838305178</v>
       </c>
       <c r="L14" t="n">
-        <v>0.002775571275715246</v>
+        <v>-0.01602175122239768</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>-1.449024114041253</v>
+        <v>-1.812859114950376</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8824816346489543</v>
+        <v>-1.058147112763505</v>
       </c>
       <c r="D15" t="n">
-        <v>1.707017101020657</v>
+        <v>0.315377654848098</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.2741118728821026</v>
+        <v>-0.08278789713652765</v>
       </c>
       <c r="F15" t="n">
-        <v>0.3131934382064296</v>
+        <v>-0.202153096702059</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2136134315026715</v>
+        <v>-0.118059937043984</v>
       </c>
       <c r="H15" t="n">
-        <v>0.09987139751909235</v>
+        <v>0.006109183673144088</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.2068746332490989</v>
+        <v>-0.05647762767469818</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.1602940326481464</v>
+        <v>0.03231403668466764</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0156300274328264</v>
+        <v>-0.04835591582396101</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.01159668224485936</v>
+        <v>-0.009112653354603163</v>
       </c>
     </row>
     <row r="16">
@@ -1755,37 +1763,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.52711166855601</v>
+        <v>-0.8888461732917488</v>
       </c>
       <c r="C16" t="n">
-        <v>0.6354196506423211</v>
+        <v>0.07781821200570219</v>
       </c>
       <c r="D16" t="n">
-        <v>-2.188972720560516</v>
+        <v>-0.5917516134974592</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.05100610639970512</v>
+        <v>-0.1243937890814983</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7604809957520723</v>
+        <v>0.1265457564087747</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.02572019054229721</v>
+        <v>-0.0152378268373352</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1068073128563993</v>
+        <v>0.02607449167463132</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.04606328351652784</v>
+        <v>0.08571189752776685</v>
       </c>
       <c r="J16" t="n">
-        <v>0.04015763165070503</v>
+        <v>-0.02675951365607826</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.01237528117126331</v>
+        <v>0.006524548672384621</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.01030937779114284</v>
+        <v>-0.01428688610912774</v>
       </c>
     </row>
     <row r="17">
@@ -1795,37 +1803,37 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-1.766360402677316</v>
+        <v>-1.524628609196013</v>
       </c>
       <c r="C17" t="n">
-        <v>-1.556817996013447</v>
+        <v>0.95267971488147</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1613393248485606</v>
+        <v>1.64304909257073</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.9766949033133883</v>
+        <v>-0.1485685106500888</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1867324265509651</v>
+        <v>0.1820296746226336</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1279556138286729</v>
+        <v>-0.1972767447624894</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.09346036185339855</v>
+        <v>-0.01581729945930283</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.0423352513904198</v>
+        <v>0.0464267746613047</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.03581418569078867</v>
+        <v>-0.04749493243565358</v>
       </c>
       <c r="K17" t="n">
-        <v>0.01723349696644758</v>
+        <v>0.01030071348477006</v>
       </c>
       <c r="L17" t="n">
-        <v>0.01077679737954257</v>
+        <v>-0.004874146905594972</v>
       </c>
     </row>
     <row r="18">
@@ -1835,37 +1843,37 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-1.791459038045157</v>
+        <v>2.194543536507407</v>
       </c>
       <c r="C18" t="n">
-        <v>-1.372051848397067</v>
+        <v>1.38548372626067</v>
       </c>
       <c r="D18" t="n">
-        <v>0.125712666013013</v>
+        <v>-1.976773392341549</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.6225748508404834</v>
+        <v>-0.03886710478072273</v>
       </c>
       <c r="F18" t="n">
-        <v>0.3819157406171066</v>
+        <v>-0.5174550263107826</v>
       </c>
       <c r="G18" t="n">
-        <v>0.01051982025399993</v>
+        <v>-0.1907489904535163</v>
       </c>
       <c r="H18" t="n">
-        <v>0.09311140838969065</v>
+        <v>0.0971829066543082</v>
       </c>
       <c r="I18" t="n">
-        <v>0.01496524993870146</v>
+        <v>-0.01265414674352174</v>
       </c>
       <c r="J18" t="n">
-        <v>0.06112854767052045</v>
+        <v>-0.01558821973023284</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.008095379732508446</v>
+        <v>-0.006264190181606877</v>
       </c>
       <c r="L18" t="n">
-        <v>0.003579361525174849</v>
+        <v>0.005704802869027132</v>
       </c>
     </row>
     <row r="19">
@@ -1875,37 +1883,37 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-2.083005955254033</v>
+        <v>-1.691944996850117</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.3514417189091709</v>
+        <v>-1.292068371420996</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.02388392862067649</v>
+        <v>0.5378610291288173</v>
       </c>
       <c r="E19" t="n">
-        <v>0.323963534247738</v>
+        <v>0.09869372079323448</v>
       </c>
       <c r="F19" t="n">
-        <v>0.1130030985400888</v>
+        <v>-0.2143415522111472</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1770154618128354</v>
+        <v>-0.06498058858893137</v>
       </c>
       <c r="H19" t="n">
-        <v>0.01966017140769568</v>
+        <v>0.033800034062642</v>
       </c>
       <c r="I19" t="n">
-        <v>0.07753009054322935</v>
+        <v>0.02275133366496494</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0923621986643153</v>
+        <v>-0.002825767628980197</v>
       </c>
       <c r="K19" t="n">
-        <v>0.01213699281891255</v>
+        <v>0.0005395987936683424</v>
       </c>
       <c r="L19" t="n">
-        <v>0.004256551138659389</v>
+        <v>0.001433864886508726</v>
       </c>
     </row>
     <row r="20">
@@ -1915,37 +1923,37 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-1.868502646737599</v>
+        <v>-1.599153871121226</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.3888128187491215</v>
+        <v>-1.212990222011216</v>
       </c>
       <c r="D20" t="n">
-        <v>0.3406174462416667</v>
+        <v>0.3785567862294375</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4788058011205533</v>
+        <v>-0.163916779867121</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.2962071817456885</v>
+        <v>-0.3996525756127634</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.01167858132934919</v>
+        <v>-0.177067662649676</v>
       </c>
       <c r="H20" t="n">
-        <v>0.09369492375599701</v>
+        <v>0.028458598520793</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.08112394425434001</v>
+        <v>-0.0221556721124623</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0520891125938056</v>
+        <v>-0.03434799975310081</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.01159171881898462</v>
+        <v>-0.007489337622519068</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.02082107063356927</v>
+        <v>0.002579306398764239</v>
       </c>
     </row>
     <row r="21">
@@ -1955,37 +1963,37 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.2104464275369029</v>
+        <v>-1.84854832205883</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.2026918065386133</v>
+        <v>-0.3757978099476215</v>
       </c>
       <c r="D21" t="n">
-        <v>0.5379437262965618</v>
+        <v>-0.19138002592106</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.4396759341422596</v>
+        <v>-0.0554476882912146</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7467793747859124</v>
+        <v>0.1374992996792788</v>
       </c>
       <c r="G21" t="n">
-        <v>0.03615355519065942</v>
+        <v>-0.08318172823576797</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.4352570386257973</v>
+        <v>-0.1048580378284781</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.08930666625041885</v>
+        <v>-0.03636228963942246</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.03508826048081359</v>
+        <v>-0.04481042946923812</v>
       </c>
       <c r="K21" t="n">
-        <v>0.000678930041159402</v>
+        <v>-0.01843592136868442</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.005420026725107554</v>
+        <v>0.00953060720494343</v>
       </c>
     </row>
     <row r="22">
@@ -1995,37 +2003,37 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3.698637645580669</v>
+        <v>-1.776383893066511</v>
       </c>
       <c r="C22" t="n">
-        <v>0.3160927543806984</v>
+        <v>-0.4739314405670856</v>
       </c>
       <c r="D22" t="n">
-        <v>-2.278239917336665</v>
+        <v>0.01300906940912093</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.3668590523824122</v>
+        <v>-0.01998207311831292</v>
       </c>
       <c r="F22" t="n">
-        <v>1.006946257441678</v>
+        <v>0.4712706375015944</v>
       </c>
       <c r="G22" t="n">
-        <v>0.06390483009610927</v>
+        <v>0.03853303619735059</v>
       </c>
       <c r="H22" t="n">
-        <v>0.1210612051939536</v>
+        <v>0.09621593812606465</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.0229340115553181</v>
+        <v>0.02136370329664621</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.007613007261524416</v>
+        <v>-0.0177595515801304</v>
       </c>
       <c r="K22" t="n">
-        <v>0.05981437518941247</v>
+        <v>0.009648052229159409</v>
       </c>
       <c r="L22" t="n">
-        <v>0.002023155896506138</v>
+        <v>0.01052459786761701</v>
       </c>
     </row>
     <row r="23">
@@ -2035,37 +2043,37 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-1.760263297550898</v>
+        <v>-0.5597942230702402</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.3490838207866293</v>
+        <v>0.1882949896369955</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1195267952145948</v>
+        <v>0.6016558962295069</v>
       </c>
       <c r="E23" t="n">
-        <v>0.5082455977074634</v>
+        <v>-0.48119487015334</v>
       </c>
       <c r="F23" t="n">
-        <v>0.05827853173618441</v>
+        <v>-0.5163500788164189</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1444849221863831</v>
+        <v>-0.1103003899082767</v>
       </c>
       <c r="H23" t="n">
-        <v>0.1579268465474851</v>
+        <v>-0.2574071582107112</v>
       </c>
       <c r="I23" t="n">
-        <v>0.02634464838467808</v>
+        <v>0.1699382685127831</v>
       </c>
       <c r="J23" t="n">
-        <v>0.000877482747832232</v>
+        <v>0.04079875473019842</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.02204062833045673</v>
+        <v>0.01888209832234048</v>
       </c>
       <c r="L23" t="n">
-        <v>0.001152680830478799</v>
+        <v>0.008878976645610982</v>
       </c>
     </row>
     <row r="24">
@@ -2075,37 +2083,37 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.08591358243060336</v>
+        <v>2.188614378948753</v>
       </c>
       <c r="C24" t="n">
-        <v>0.8664606076354067</v>
+        <v>1.429814662901902</v>
       </c>
       <c r="D24" t="n">
-        <v>-1.211431968226085</v>
+        <v>-1.98890761918643</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.6615093061522573</v>
+        <v>-0.02218777904216162</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.232650256684238</v>
+        <v>-0.4450594681114973</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.2608629757143615</v>
+        <v>-0.1583388302148715</v>
       </c>
       <c r="H24" t="n">
-        <v>0.02901446351202978</v>
+        <v>0.1181678268367057</v>
       </c>
       <c r="I24" t="n">
-        <v>0.06131022180476729</v>
+        <v>-0.0278469540987407</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.1184986782225678</v>
+        <v>-0.02416264098507272</v>
       </c>
       <c r="K24" t="n">
-        <v>0.02032806454059989</v>
+        <v>-0.001516259597413297</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.01118408422866394</v>
+        <v>0.02394111815727526</v>
       </c>
     </row>
     <row r="25">
@@ -2115,73 +2123,157 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.4842427320505819</v>
+        <v>-1.588176757884407</v>
       </c>
       <c r="C25" t="n">
-        <v>0.502418322447811</v>
+        <v>-0.339893523328794</v>
       </c>
       <c r="D25" t="n">
-        <v>0.26952880933892</v>
+        <v>-0.1868244476217634</v>
       </c>
       <c r="E25" t="n">
-        <v>1.221875240673646</v>
+        <v>-0.09778182043690695</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.074994268573092</v>
+        <v>0.2344612145171157</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2611254075763628</v>
+        <v>-0.03075961694488372</v>
       </c>
       <c r="H25" t="n">
-        <v>0.05424727847481029</v>
+        <v>0.1018677464829768</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.2696468937717132</v>
+        <v>0.01675825163002015</v>
       </c>
       <c r="J25" t="n">
-        <v>0.09017821614327685</v>
+        <v>-0.02375215527575084</v>
       </c>
       <c r="K25" t="n">
-        <v>0.04626666979542147</v>
+        <v>0.006950933992989713</v>
       </c>
       <c r="L25" t="n">
-        <v>-0.000208852930009719</v>
+        <v>-0.006097904691384199</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Vancomycin HCl</t>
+        </is>
+      </c>
       <c r="B26" t="n">
-        <v>10.1626835016694</v>
+        <v>-0.8668350123925005</v>
       </c>
       <c r="C26" t="n">
-        <v>-1.632331310853753</v>
+        <v>0.2223404801442957</v>
       </c>
       <c r="D26" t="n">
-        <v>2.138576046792243</v>
+        <v>-0.4358408789773653</v>
       </c>
       <c r="E26" t="n">
-        <v>0.5182809371873446</v>
+        <v>0.1773503386380494</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2617245805010905</v>
+        <v>1.019502115479428</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.01593302227506316</v>
+        <v>0.1654574101445727</v>
       </c>
       <c r="H26" t="n">
-        <v>0.04942922908481354</v>
+        <v>-0.01076908647392176</v>
       </c>
       <c r="I26" t="n">
-        <v>0.171540271517642</v>
+        <v>-0.01797278777000173</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.01023795874024229</v>
+        <v>-0.03634910718194219</v>
       </c>
       <c r="K26" t="n">
-        <v>0.007845217586300537</v>
+        <v>0.02283067523638826</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.005402759472677358</v>
+        <v>0.02028019805164913</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Naringenin</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>6.337189904968314</v>
+      </c>
+      <c r="C27" t="n">
+        <v>-0.1216064724641592</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.8272937400916386</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-2.512326712223067</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-0.1529435912778404</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.3692318088745061</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.02228879231628399</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-0.0893156002422088</v>
+      </c>
+      <c r="J27" t="n">
+        <v>-0.05142027785367383</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-0.01138809159956398</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.001554517662881983</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ritonavir</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>-0.08718793964779278</v>
+      </c>
+      <c r="C28" t="n">
+        <v>-0.1889905664547802</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.3491096822733129</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1.268053297941188</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-0.4706557477228569</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.395319895474659</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.04854137038544658</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0.01418823307251272</v>
+      </c>
+      <c r="J28" t="n">
+        <v>-0.0233787443145742</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.02324295801132854</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.006910913263670514</v>
       </c>
     </row>
   </sheetData>
@@ -2195,7 +2287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2206,318 +2298,274 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>descriptor_source</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>smiles</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>smiles_source</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>molecular_weight</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>logp</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rotatable_bond_count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>hbond_acceptor_count</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>hbond_donor_count</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>heavy_atom_count</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>tpsa</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>complexity</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Formal charge</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>number_of_rings</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>aromatic_ring_count</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>saturated_ring_count</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>fraction_csp3</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>heteroatom_count</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>formal_charge</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>atom_count</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>amide_bond_count</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>defined_atom_stereocenter_count</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>defined_bond_stereocenter_count</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>number_of_rings</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>number_of_rings_calc</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>smiles</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>smiles_source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cathelicidin (LL37)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4493</v>
-      </c>
-      <c r="C2" t="n">
-        <v>-18.3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>171</v>
+          <t>(CRA)- H P 228</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual backup</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>69</v>
+        <v>942.1</v>
       </c>
       <c r="F2" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H2" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" t="n">
         <v>68</v>
       </c>
-      <c r="G2" t="n">
-        <v>318</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1890</v>
-      </c>
-      <c r="I2" t="n">
-        <v>10600</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
       <c r="K2" t="n">
-        <v>39</v>
+        <v>392</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1820</v>
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>6</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bortezomib</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>384.2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="D3" t="n">
-        <v>9</v>
+          <t>Glatiramer acetate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manual backup</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4</v>
-      </c>
+        <v>623.7</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="H3" t="n">
-        <v>124</v>
+        <v>18</v>
       </c>
       <c r="I3" t="n">
-        <v>500</v>
+        <v>12</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>374</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>2</v>
-      </c>
+        <v>519</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>4</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(CRA)- H P 228</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>942.1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="D4" t="n">
-        <v>29</v>
+          <t>Granulocyte-Colony Stimulating Factor</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manual backup</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>727.8</v>
       </c>
       <c r="F4" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>22</v>
+      </c>
+      <c r="H4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I4" t="n">
         <v>12</v>
       </c>
-      <c r="G4" t="n">
-        <v>68</v>
-      </c>
-      <c r="H4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1820</v>
-      </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>359</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1170</v>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Glatiramer acetate</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>623.7</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
-        <v>13</v>
-      </c>
-      <c r="E5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F5" t="n">
-        <v>12</v>
-      </c>
-      <c r="G5" t="n">
-        <v>43</v>
-      </c>
-      <c r="H5" t="n">
-        <v>374</v>
-      </c>
-      <c r="I5" t="n">
-        <v>519</v>
-      </c>
-      <c r="J5" t="n">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" t="n">
         <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Granulocyte‑Colony Stimulating Factor</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>727.8</v>
-      </c>
-      <c r="C6" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E6" t="n">
-        <v>13</v>
-      </c>
-      <c r="F6" t="n">
-        <v>12</v>
-      </c>
-      <c r="G6" t="n">
-        <v>50</v>
-      </c>
-      <c r="H6" t="n">
-        <v>359</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1170</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new API descriptors to PCA analysis
</commit_message>
<xml_diff>
--- a/api_pca_results.xlsx
+++ b/api_pca_results.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,13 +448,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7396822596646899</v>
+        <v>0.6829876176034376</v>
       </c>
       <c r="C2" t="n">
-        <v>73.96822596646899</v>
+        <v>68.29876176034377</v>
       </c>
       <c r="D2" t="n">
-        <v>73.96822596646899</v>
+        <v>68.29876176034377</v>
       </c>
     </row>
     <row r="3">
@@ -464,13 +464,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1184354314738571</v>
+        <v>0.1021743313291748</v>
       </c>
       <c r="C3" t="n">
-        <v>11.84354314738571</v>
+        <v>10.21743313291748</v>
       </c>
       <c r="D3" t="n">
-        <v>85.81176911385471</v>
+        <v>78.51619489326124</v>
       </c>
     </row>
     <row r="4">
@@ -480,13 +480,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.07885988345682321</v>
+        <v>0.09965817367375222</v>
       </c>
       <c r="C4" t="n">
-        <v>7.885988345682321</v>
+        <v>9.965817367375223</v>
       </c>
       <c r="D4" t="n">
-        <v>93.69775745953703</v>
+        <v>88.48201226063645</v>
       </c>
     </row>
     <row r="5">
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04501137305239598</v>
+        <v>0.05347396723869859</v>
       </c>
       <c r="C5" t="n">
-        <v>4.501137305239598</v>
+        <v>5.347396723869859</v>
       </c>
       <c r="D5" t="n">
-        <v>98.19889476477664</v>
+        <v>93.82940898450632</v>
       </c>
     </row>
     <row r="6">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01325358807765344</v>
+        <v>0.03989212465983037</v>
       </c>
       <c r="C6" t="n">
-        <v>1.325358807765344</v>
+        <v>3.989212465983037</v>
       </c>
       <c r="D6" t="n">
-        <v>99.52425357254198</v>
+        <v>97.81862145048935</v>
       </c>
     </row>
     <row r="7">
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00282747772541384</v>
+        <v>0.01171960059564808</v>
       </c>
       <c r="C7" t="n">
-        <v>0.282747772541384</v>
+        <v>1.171960059564808</v>
       </c>
       <c r="D7" t="n">
-        <v>99.80700134508336</v>
+        <v>98.99058151005416</v>
       </c>
     </row>
     <row r="8">
@@ -544,13 +544,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0009842637891835004</v>
+        <v>0.005749016023262258</v>
       </c>
       <c r="C8" t="n">
-        <v>0.09842637891835004</v>
+        <v>0.5749016023262259</v>
       </c>
       <c r="D8" t="n">
-        <v>99.90542772400171</v>
+        <v>99.56548311238038</v>
       </c>
     </row>
     <row r="9">
@@ -560,13 +560,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0006920096145600679</v>
+        <v>0.002160218363405858</v>
       </c>
       <c r="C9" t="n">
-        <v>0.06920096145600679</v>
+        <v>0.2160218363405858</v>
       </c>
       <c r="D9" t="n">
-        <v>99.97462868545772</v>
+        <v>99.78150494872096</v>
       </c>
     </row>
     <row r="10">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0001967862565253606</v>
+        <v>0.0009948917211693689</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01967862565253605</v>
+        <v>0.09948917211693689</v>
       </c>
       <c r="D10" t="n">
-        <v>99.99430731111025</v>
+        <v>99.88099412083791</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.039334361622885e-05</v>
+        <v>0.0005113746506266259</v>
       </c>
       <c r="C11" t="n">
-        <v>0.004039334361622885</v>
+        <v>0.05113746506266259</v>
       </c>
       <c r="D11" t="n">
-        <v>99.99834664547187</v>
+        <v>99.93213158590058</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,125 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.653354528114542e-05</v>
+        <v>0.000306998414899189</v>
       </c>
       <c r="C12" t="n">
-        <v>0.001653354528114542</v>
+        <v>0.0306998414899189</v>
       </c>
       <c r="D12" t="n">
-        <v>99.99999999999999</v>
+        <v>99.9628314273905</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.0002347067736501655</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.02347067736501655</v>
+      </c>
+      <c r="D13" t="n">
+        <v>99.98630210475551</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PC13</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8.031444037406305e-05</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.008031444037406306</v>
+      </c>
+      <c r="D14" t="n">
+        <v>99.99433354879291</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PC14</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.51076004710023e-05</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.003510760047100229</v>
+      </c>
+      <c r="D15" t="n">
+        <v>99.99784430884002</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PC15</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.813830806432101e-05</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.001813830806432101</v>
+      </c>
+      <c r="D16" t="n">
+        <v>99.99965813964644</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PC16</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3.418603535405527e-06</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0003418603535405527</v>
+      </c>
+      <c r="D17" t="n">
+        <v>99.99999999999997</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PC17</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6.098902137787327e-35</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6.098902137787327e-33</v>
+      </c>
+      <c r="D18" t="n">
+        <v>99.99999999999997</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PC18</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.651066957992938e-37</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1.651066957992938e-35</v>
+      </c>
+      <c r="D19" t="n">
+        <v>99.99999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -628,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +799,41 @@
           <t>PC11</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>PC13</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>PC14</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>PC15</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>PC16</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>PC17</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>PC18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -695,37 +842,58 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3480441041852776</v>
+        <v>0.292555911505707</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04840257616094605</v>
+        <v>0.01209496908042476</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0395850795322399</v>
+        <v>0.006114071157475818</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.07044592927863616</v>
+        <v>0.05021254613209371</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1227340622519716</v>
+        <v>-0.002679372930503698</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3489385360214914</v>
+        <v>0.05083684903521189</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.08294085362001047</v>
+        <v>0.1563538441034655</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.4144835056110443</v>
+        <v>-0.005121518871821546</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.1571621003056827</v>
+        <v>-0.08670351957530033</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.1109574816719508</v>
+        <v>-0.1149450627430896</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7193635260404461</v>
+        <v>-0.2066868790709916</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-0.2004029363581004</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-0.03183958071116434</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-0.2734289408792462</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-0.2278569511049212</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.8082914972436338</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-0</v>
       </c>
     </row>
     <row r="3">
@@ -735,37 +903,58 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.2717844848700969</v>
+        <v>-0.2241232219669497</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4600596601471946</v>
+        <v>0.2667638534404871</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.1555368520902943</v>
+        <v>0.3430698658226735</v>
       </c>
       <c r="E3" t="n">
-        <v>0.223475675715559</v>
+        <v>0.01026657043827786</v>
       </c>
       <c r="F3" t="n">
-        <v>0.720643180761425</v>
+        <v>0.2375212462789646</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1723064116028518</v>
+        <v>0.2276669810117067</v>
       </c>
       <c r="H3" t="n">
-        <v>0.278423950860016</v>
+        <v>0.6678380905262079</v>
       </c>
       <c r="I3" t="n">
-        <v>0.08087387598281544</v>
+        <v>0.02869388608615136</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.0003515313889551203</v>
+        <v>0.1185639113567169</v>
       </c>
       <c r="K3" t="n">
-        <v>0.08374251800218749</v>
+        <v>-0.3539327146075258</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01599081962926729</v>
+        <v>0.1238665999499238</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-0.06574464320072705</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1607521972011305</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.009907394569537209</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.1378435832993911</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-0.04233795658632378</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-8.467780417813657e-17</v>
+      </c>
+      <c r="S3" t="n">
+        <v>8.053890807863828e-18</v>
       </c>
     </row>
     <row r="4">
@@ -775,37 +964,58 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3304195706146875</v>
+        <v>0.2722901440003537</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.1619310960143837</v>
+        <v>-0.05957395279525762</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1621051707555164</v>
+        <v>-0.1969698134079306</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1430348306248074</v>
+        <v>0.07208109221823868</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4918425292955053</v>
+        <v>0.2411553208873852</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.4197663500681541</v>
+        <v>0.09588486732070536</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.5448147945544466</v>
+        <v>0.3469222669147973</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2768259899287904</v>
+        <v>0.3635630111396347</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.1478079368384611</v>
+        <v>-0.2647077290243893</v>
       </c>
       <c r="K4" t="n">
-        <v>0.04687917767652454</v>
+        <v>0.5561124727170722</v>
       </c>
       <c r="L4" t="n">
-        <v>0.04744136918318019</v>
+        <v>0.3243537849565395</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.2276205532438263</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1015348738657216</v>
+      </c>
+      <c r="O4" t="n">
+        <v>-0.07197467541228712</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.07841652423921809</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.02113569206015313</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1.443913504521839e-16</v>
+      </c>
+      <c r="S4" t="n">
+        <v>6.150081859228522e-18</v>
       </c>
     </row>
     <row r="5">
@@ -815,37 +1025,58 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3436447736645724</v>
+        <v>0.2898054787715753</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1092177379593841</v>
+        <v>0.04756100127849142</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.01671977112053451</v>
+        <v>0.06205077496719423</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1250756199421833</v>
+        <v>0.0254066456542625</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.09715381142050872</v>
+        <v>-0.06115884665335814</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5801949996531719</v>
+        <v>0.007601193255699588</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.03806377030439162</v>
+        <v>-0.1189238812550072</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7014635639584008</v>
+        <v>-0.2261060331339345</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.05587379391002843</v>
+        <v>-0.531871899860854</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.07671459258153267</v>
+        <v>-0.3730571799596994</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.07405539392833699</v>
+        <v>0.6030011046023132</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-0.1340860837545559</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-0.1235729227257736</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.1278686198975868</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.04807386741652576</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-0.05108222387023936</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.049624119736836e-17</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-6.835317499249891e-18</v>
       </c>
     </row>
     <row r="6">
@@ -855,37 +1086,58 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3463977141952448</v>
+        <v>0.2876214665551332</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.09687788400027632</v>
+        <v>0.001787972518615037</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02498892564205073</v>
+        <v>-0.1366140040501975</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.04766242489352817</v>
+        <v>0.01167532492100639</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05371991268105927</v>
+        <v>0.03294395993648866</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.3480743404589615</v>
+        <v>-0.05965352134817738</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6877572692733405</v>
+        <v>-0.06907502934928669</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1038228181389322</v>
+        <v>0.135078059703383</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.4093847889325154</v>
+        <v>0.3064766457749984</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.3037746705301073</v>
+        <v>-0.4319076220979891</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.00462338257495204</v>
+        <v>0.09769264231103399</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.6700097985733899</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.2431406035452383</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-0.0003113062376722247</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-0.2695498369770317</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.01029714629289662</v>
+      </c>
+      <c r="R6" t="n">
+        <v>6.630346260352756e-17</v>
+      </c>
+      <c r="S6" t="n">
+        <v>5.386808643152657e-20</v>
       </c>
     </row>
     <row r="7">
@@ -895,37 +1147,58 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3483766950177057</v>
+        <v>0.2925300997828106</v>
       </c>
       <c r="C7" t="n">
-        <v>0.04596915079947084</v>
+        <v>0.01230617664597992</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03698802635088281</v>
+        <v>0.003162235340474906</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.04830070664152148</v>
+        <v>0.04364090383615486</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1439002603103246</v>
+        <v>0.01760419526273376</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2731614965110287</v>
+        <v>0.0463947277879276</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.08886311896821164</v>
+        <v>0.1721191329674826</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.4729655601714178</v>
+        <v>0.05992799386784303</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.2963297862608043</v>
+        <v>-0.05706901328501741</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1522207217869724</v>
+        <v>-0.09095786880484362</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.6594841845765869</v>
+        <v>-0.2773625019867743</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-0.01500630001870578</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-0.3714118780495689</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-0.1531105925557019</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-0.1143650729856703</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-0.3369377870260649</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.7071067810630349</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-1.321641819895752e-05</v>
       </c>
     </row>
     <row r="8">
@@ -935,37 +1208,58 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.348590672645173</v>
+        <v>0.2903546916224534</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.06761960552236101</v>
+        <v>-0.01771261568883749</v>
       </c>
       <c r="D8" t="n">
-        <v>0.05751176825984187</v>
+        <v>-0.09979708694814132</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.03752206718068614</v>
+        <v>0.03322466957931148</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.003404444973988396</v>
+        <v>0.0343994849776547</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.07865818230381347</v>
+        <v>-0.04539836251474381</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3108627720143484</v>
+        <v>-0.08726367204004909</v>
       </c>
       <c r="I8" t="n">
-        <v>0.04223580640118429</v>
+        <v>0.0008027374237403433</v>
       </c>
       <c r="J8" t="n">
-        <v>0.319779170939097</v>
+        <v>0.03046236323845826</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8046427127606141</v>
+        <v>-0.20284996672231</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1219417207477423</v>
+        <v>-0.1424935577357676</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0896259748230312</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-0.03958765708207483</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-0.0228025381595663</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.8983632737776938</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.117898882057618</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-1.8402832578503e-16</v>
+      </c>
+      <c r="S8" t="n">
+        <v>2.199632688866561e-17</v>
       </c>
     </row>
     <row r="9">
@@ -975,37 +1269,58 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.3468107306911331</v>
+        <v>0.2906254158479507</v>
       </c>
       <c r="C9" t="n">
-        <v>0.06927662248080196</v>
+        <v>0.09044120257993998</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.01755600620588045</v>
+        <v>-0.01392105394310344</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1275281437178474</v>
+        <v>0.04903739620042843</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1881477230962233</v>
+        <v>-0.01348715058034322</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.06661008130287661</v>
+        <v>0.02352061957993946</v>
       </c>
       <c r="H9" t="n">
-        <v>0.05113272283554106</v>
+        <v>0.08535357848632902</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.1243647453691872</v>
+        <v>0.1275257459639451</v>
       </c>
       <c r="J9" t="n">
-        <v>0.759887735282643</v>
+        <v>-0.0405877293251965</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.44694779502802</v>
+        <v>0.02708399664020491</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.1524536331968943</v>
+        <v>-0.2901617295126436</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-0.1585851917855154</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.1664438188662546</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.8561907871819988</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-0.08346089824307926</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.03193263451326364</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-6.833926941232111e-16</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-1.115384314749725e-17</v>
       </c>
     </row>
     <row r="10">
@@ -1015,37 +1330,58 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2574287906374266</v>
+        <v>0.2113393296861263</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1679571146662453</v>
+        <v>-0.02642434937081405</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1719811428985963</v>
+        <v>0.1899461241907346</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8818659623884528</v>
+        <v>-0.3253798110098939</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.3022065344352616</v>
+        <v>0.6209229882480882</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.01121982199923165</v>
+        <v>-0.5386027681463373</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.01328354625147483</v>
+        <v>-0.002739919114523326</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.03539646903607532</v>
+        <v>-0.2808466423828462</v>
       </c>
       <c r="J10" t="n">
-        <v>0.04586766351738255</v>
+        <v>0.1730645369575851</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.05704346125158385</v>
+        <v>0.1185275942017392</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.003728369820071527</v>
+        <v>0.04818420984629731</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-0.08495738097378254</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-0.03696007426439404</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.02688253688717646</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-0.05030568765392397</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-0.002503558755023043</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.714427404414166e-17</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-2.741932572210066e-18</v>
       </c>
     </row>
     <row r="11">
@@ -1055,37 +1391,58 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01156641681075643</v>
+        <v>0.01704800663221426</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6381336580720642</v>
+        <v>-0.01387046717142662</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7294267861505931</v>
+        <v>0.4504890553993778</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.04758114842870974</v>
+        <v>0.822713741140544</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.185448902484309</v>
+        <v>0.209818547408313</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1512893948276761</v>
+        <v>-0.09683489936000467</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.02287883588383523</v>
+        <v>-0.2320534188698802</v>
       </c>
       <c r="I11" t="n">
-        <v>0.000251234724914865</v>
+        <v>0.05410169139493414</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.02211404971593781</v>
+        <v>0.03058124496601571</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.004261008262157466</v>
+        <v>0.07565546440445299</v>
       </c>
       <c r="L11" t="n">
-        <v>0.003712457602717819</v>
+        <v>-0.00433322739309798</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.04837677753442463</v>
+      </c>
+      <c r="N11" t="n">
+        <v>-0.00474066212776272</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-0.0171023253864479</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-0.01270101257478836</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.006910389930513018</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-8.131843795844208e-18</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-1.966531034519136e-19</v>
       </c>
     </row>
     <row r="12">
@@ -1095,37 +1452,485 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1678555032098235</v>
+        <v>0.1459841024642718</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5399609235365636</v>
+        <v>0.4629768702051163</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.6167935998218748</v>
+        <v>0.3741542627706067</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.3267500277830358</v>
+        <v>-0.2444295012656766</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1718646691793672</v>
+        <v>-0.2978201095163178</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.3260537451065727</v>
+        <v>-0.2601646688682381</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1909766476838945</v>
+        <v>-0.1780144081675542</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0002333491717852951</v>
+        <v>0.5649614841048378</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.1124396452737646</v>
+        <v>0.08447459508722199</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0815984312712674</v>
+        <v>0.0591986944331687</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0380155786551334</v>
+        <v>0.1239439324323447</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-0.1277578412065113</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-0.003626734359654995</v>
+      </c>
+      <c r="O12" t="n">
+        <v>-0.117601022123942</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.03368504729142317</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>-0.00695287102821277</v>
+      </c>
+      <c r="R12" t="n">
+        <v>3.913531433406315e-17</v>
+      </c>
+      <c r="S12" t="n">
+        <v>2.780358255201802e-18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>aromatic_ring_count</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1104316274010218</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6860366211456691</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.03349114111918803</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-0.04231802142345038</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.05453306656975156</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.3499340246405621</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.1666666869021749</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0.4434284523013569</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-0.01528236356806106</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.2816679927101474</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-0.08661219746532382</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.2727373363763821</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-0.03691371423464603</v>
+      </c>
+      <c r="O13" t="n">
+        <v>-0.01580886981242715</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-0.0007407421498174043</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.03662044978759676</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1.066883942035045e-16</v>
+      </c>
+      <c r="S13" t="n">
+        <v>-9.789657253989965e-19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>saturated_ring_count</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1574095132803282</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-0.2789863420209398</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.4614046606155013</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.06770088913245997</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.5312051927363706</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-0.1703373673386153</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3183741187018993</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-0.3471101729189591</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-0.02308352528657881</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.2190299056085784</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.0245748827045706</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.298315334262033</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.06117146416031094</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.03559201754943536</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.05788049477251483</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.02020059752532793</v>
+      </c>
+      <c r="R14" t="n">
+        <v>2.471024559029048e-17</v>
+      </c>
+      <c r="S14" t="n">
+        <v>2.520239071327296e-18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fraction_csp3</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.130560220826499</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-0.3842805117841873</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.4419636458202623</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.3335385439400238</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.2122697119232503</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.6048769216126003</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.3084525937633167</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.1434479931920605</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.02604490905255877</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.01271663244765648</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-0.0209227836191545</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.01743729010933593</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.0158810577565866</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.01236076998097736</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.0009329300448181222</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.007752628782013518</v>
+      </c>
+      <c r="R15" t="n">
+        <v>-1.223742408148006e-17</v>
+      </c>
+      <c r="S15" t="n">
+        <v>2.929999722519866e-19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>heteroatom_count</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2915584688705216</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.002972639682442009</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.05664805820759385</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.05850826404176694</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.0508321875636851</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.03775455538641893</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.04985801051077755</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0.1442747398201829</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-0.05102601931783927</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.001407626665510237</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-0.1342262798213341</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-0.3367260262806848</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.7376709754439493</v>
+      </c>
+      <c r="O16" t="n">
+        <v>-0.3233140063470171</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.02380177920346433</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-0.312695662330911</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-2.364482981367199e-16</v>
+      </c>
+      <c r="S16" t="n">
+        <v>2.600679416457928e-17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>formal_charge</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1.869083786296133e-05</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.9999999998253263</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>atom_count</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.2925300997828106</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.01230617664597989</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.003162235340474948</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.04364090383615488</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.01760419526273392</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.04639472778792766</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.1721191329674828</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.05992799386784295</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-0.05706901328501703</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-0.09095786880484345</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-0.2773625019867738</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-0.01500630001870575</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-0.3714118780495696</v>
+      </c>
+      <c r="O18" t="n">
+        <v>-0.1531105925557026</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-0.1143650729856704</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>-0.336937787026065</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-0.7071067810630348</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1.321641819893289e-05</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>amide_bond_count</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2794930408770562</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.05178835273945064</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.1386128557567501</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1433774606307089</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.1659779675112449</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.199820489513011</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.06174272769044182</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0.1211035030387539</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.6930940089354309</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.1317662074658238</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.4011947542246556</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-0.3165978835136729</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-0.1799077736315904</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.04574590700776476</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.006099585737357627</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>-0.006786806505451783</v>
+      </c>
+      <c r="R19" t="n">
+        <v>5.431918717100666e-16</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-5.634533827638617e-18</v>
       </c>
     </row>
   </sheetData>
@@ -1139,7 +1944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1203,6 +2008,41 @@
           <t>PC11</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>PC13</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>PC14</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>PC15</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>PC16</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>PC17</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>PC18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1211,37 +2051,58 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4994196562552905</v>
+        <v>0.8060893486564648</v>
       </c>
       <c r="C2" t="n">
-        <v>2.472678638941129</v>
+        <v>3.109116747481643</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3682638423581847</v>
+        <v>1.280938698223757</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.4841451139010026</v>
+        <v>1.363016174111248</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3303438807789143</v>
+        <v>0.589611366955669</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1065663275750653</v>
+        <v>0.7413091839353565</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1022095167285055</v>
+        <v>-0.4066551696087257</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1891933688824013</v>
+        <v>-0.3325234916517621</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1127146836797746</v>
+        <v>-0.04168547218930086</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.03235178406878325</v>
+        <v>0.009413196171431272</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0006366664350142242</v>
+        <v>0.05444071131203111</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-0.05295420387415754</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.02438832283379606</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.04628052117523295</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-0.0161108089732519</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.004074476258075131</v>
+      </c>
+      <c r="R2" t="n">
+        <v>3.288361233392808e-18</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2.429449265480645e-19</v>
       </c>
     </row>
     <row r="3">
@@ -1251,37 +2112,58 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.518194283051294</v>
+        <v>3.006371808474067</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.7846411752384059</v>
+        <v>-0.2171201598511673</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01962216128453597</v>
+        <v>-0.7481217262986636</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08981860151928035</v>
+        <v>-0.302885353827357</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.4004249035431454</v>
+        <v>0.1748757342037966</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1012289689359072</v>
+        <v>0.1840095657279615</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1081782169677781</v>
+        <v>-0.5139790821498222</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.0800810654884255</v>
+        <v>-0.2911392182700051</v>
       </c>
       <c r="J3" t="n">
-        <v>0.09776920707564295</v>
+        <v>0.1244395839170855</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0523890689825259</v>
+        <v>0.01172393934693383</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.02490192027989758</v>
+        <v>-0.1270033120166539</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-0.06868326802888723</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-0.0968338443379058</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.000232375253969917</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.02561222057291286</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-0.009873073019003418</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-2.984349716976627e-17</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-2.516781312125146e-20</v>
       </c>
     </row>
     <row r="4">
@@ -1291,37 +2173,58 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-1.84364081844942</v>
+        <v>-2.256617973845516</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.296221089181179</v>
+        <v>-1.538472918442241</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5322411559964286</v>
+        <v>-0.8596482247773115</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01124748356239265</v>
+        <v>-0.1438192032433255</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2200723542953316</v>
+        <v>0.1873183420424393</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.09930281003495653</v>
+        <v>0.3760122196969505</v>
       </c>
       <c r="H4" t="n">
-        <v>0.106160684629904</v>
+        <v>-0.4435173314846487</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.09675655750282203</v>
+        <v>0.2237897541390827</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01005955453971012</v>
+        <v>0.09189049516590878</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.01391325337486565</v>
+        <v>-0.08625118735339121</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0005222115222033951</v>
+        <v>-0.1326646252164199</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.01145106103936953</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.05066483196673446</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.01051372623262077</v>
+      </c>
+      <c r="P4" t="n">
+        <v>-0.01662877151874494</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.003243314685652564</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2.531948349518272e-18</v>
+      </c>
+      <c r="S4" t="n">
+        <v>8.747132786346075e-19</v>
       </c>
     </row>
     <row r="5">
@@ -1331,37 +2234,58 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11.23039066909353</v>
+        <v>12.77283914641589</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.422663573121028</v>
+        <v>-0.3655072045019341</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6659723395951535</v>
+        <v>-2.405830699539361</v>
       </c>
       <c r="E5" t="n">
-        <v>1.317476102034821</v>
+        <v>0.06481190252167589</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4962108703658131</v>
+        <v>2.014236966984853</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2542860730991719</v>
+        <v>-0.2165048501057488</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.03935772062311443</v>
+        <v>0.2310984980022156</v>
       </c>
       <c r="I5" t="n">
-        <v>0.05289304574184379</v>
+        <v>0.1521768857782673</v>
       </c>
       <c r="J5" t="n">
-        <v>0.004977187612214575</v>
+        <v>-0.04137447198101765</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.007591791906127566</v>
+        <v>0.03637871794974707</v>
       </c>
       <c r="L5" t="n">
-        <v>0.002280224059648944</v>
+        <v>0.0266913101852161</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.0151968072412153</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.01956859643833346</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.007775384306031734</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.0006017871373042573</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.0006184965974638201</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-1.3172129212778e-17</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2.143049361653997e-20</v>
       </c>
     </row>
     <row r="6">
@@ -1371,37 +2295,58 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.3544797707292202</v>
+        <v>-0.1377555482349118</v>
       </c>
       <c r="C6" t="n">
-        <v>3.370109261913631</v>
+        <v>-1.485878083901734</v>
       </c>
       <c r="D6" t="n">
-        <v>2.518330746021151</v>
+        <v>3.81372352227048</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9202304622335878</v>
+        <v>2.413245890988593</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.2547031258630256</v>
+        <v>1.191065058134873</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.04824045660832674</v>
+        <v>-0.4970510074769629</v>
       </c>
       <c r="H6" t="n">
-        <v>0.02520846413451666</v>
+        <v>0.1384598443174148</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.1379540081717562</v>
+        <v>0.1408748173898609</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.03024812048719854</v>
+        <v>0.1362892353152107</v>
       </c>
       <c r="K6" t="n">
-        <v>0.009140420378840669</v>
+        <v>-0.0572939354162253</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.0004854918345328356</v>
+        <v>-0.04319132543526153</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-0.02304631017714869</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-0.01185311745226131</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-0.004298381272866554</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.006188184079570742</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.002659444604536469</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-1.518131082280446e-17</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1.161544165704909e-19</v>
       </c>
     </row>
     <row r="7">
@@ -1411,37 +2356,58 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-1.853105967891027</v>
+        <v>-2.520551066117406</v>
       </c>
       <c r="C7" t="n">
-        <v>-1.261267475422086</v>
+        <v>-0.782521544794057</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5249731116318999</v>
+        <v>-1.690026416550172</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.008198063287445425</v>
+        <v>0.5110938337593499</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2728112856173099</v>
+        <v>-0.2582207626623423</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1000397417737514</v>
+        <v>-0.7997779715525806</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.05890771896352544</v>
+        <v>0.1242074306034454</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04261231045161718</v>
+        <v>-0.1489665433363107</v>
       </c>
       <c r="J7" t="n">
-        <v>0.06910302467520685</v>
+        <v>-0.1425208570586057</v>
       </c>
       <c r="K7" t="n">
-        <v>0.004870169613261754</v>
+        <v>-0.08714045425602941</v>
       </c>
       <c r="L7" t="n">
-        <v>0.03630489053742018</v>
+        <v>0.03924530311401394</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-0.2084168580701999</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-0.002222200885448973</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-0.007411270505783404</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.001749930623049917</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.01522092085211142</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-1.300025473750682e-17</v>
+      </c>
+      <c r="S7" t="n">
+        <v>2.182277704842821e-19</v>
       </c>
     </row>
     <row r="8">
@@ -1451,37 +2417,58 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.2984695197554383</v>
+        <v>-0.1110681882476334</v>
       </c>
       <c r="C8" t="n">
-        <v>0.03708503297232664</v>
+        <v>-2.119347807969487</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.430342098334104</v>
+        <v>1.850866062572223</v>
       </c>
       <c r="E8" t="n">
-        <v>1.388665331647193</v>
+        <v>-1.555210541032255</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.1250990702351577</v>
+        <v>0.5678997101193722</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4767666924061776</v>
+        <v>0.08255300464111467</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.02225510521777503</v>
+        <v>0.3274088696345455</v>
       </c>
       <c r="I8" t="n">
-        <v>0.04654889665497481</v>
+        <v>-0.2982305373676555</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.02119042365839661</v>
+        <v>-0.1063034626322029</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.04258423862270947</v>
+        <v>-0.05730418572840406</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.01235764574545984</v>
+        <v>0.07493495103590057</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-0.0004581766595494357</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.02432707836140304</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.03207062952949603</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-0.02042433010294729</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>-0.01265667150165609</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-3.950071085101069e-17</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-2.273249148359293e-19</v>
       </c>
     </row>
     <row r="9">
@@ -1491,37 +2478,58 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.5137953612039901</v>
+        <v>-0.7197201034718054</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.1157396809219698</v>
+        <v>-0.0157058766724529</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.5345292425711552</v>
+        <v>0.1577826941065335</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.07820120817246806</v>
+        <v>-0.6178350029706348</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.2793055195670694</v>
+        <v>-0.1732983753821617</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0314415688383424</v>
+        <v>-0.105066332917976</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.06297643852929412</v>
+        <v>-0.2774923765000177</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1044781732223136</v>
+        <v>0.1383212268153416</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.02246166071738499</v>
+        <v>-0.18957610736386</v>
       </c>
       <c r="K9" t="n">
-        <v>0.01180378141762061</v>
+        <v>-0.01797374434444253</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.01550128915383261</v>
+        <v>0.02681660987362441</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.07240467751889153</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-0.03252975859314797</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.01624165483340757</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.01033509912083287</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.005876269024626171</v>
+      </c>
+      <c r="R9" t="n">
+        <v>3.137429028865497e-17</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.579289617549187e-18</v>
       </c>
     </row>
     <row r="10">
@@ -1531,37 +2539,58 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.230498008401778</v>
+        <v>-1.497044702126997</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.7368187691394492</v>
+        <v>-0.1732047840846914</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1154506504990819</v>
+        <v>-0.7439381983135327</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0003106754836107111</v>
+        <v>-0.1183356467910958</v>
       </c>
       <c r="F10" t="n">
-        <v>0.08011496636265077</v>
+        <v>0.1827400499279593</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.03446608198497465</v>
+        <v>0.3684242877008134</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.05033907337489325</v>
+        <v>-0.1485283119861725</v>
       </c>
       <c r="I10" t="n">
-        <v>0.001727926765278782</v>
+        <v>0.001724841371221122</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.05056704847719513</v>
+        <v>0.01989830242778603</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.01314870591834223</v>
+        <v>0.09288209036009182</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.00802726255141864</v>
+        <v>0.005846652868646919</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.0354575662888072</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-0.04942313076411104</v>
+      </c>
+      <c r="O10" t="n">
+        <v>-0.03984858039754566</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-0.04606652613246146</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-0.001472202868048293</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2.549981549646863e-17</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-1.410793356986903e-18</v>
       </c>
     </row>
     <row r="11">
@@ -1571,37 +2600,58 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-1.641610848838819</v>
+        <v>-1.969130657614917</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.2510166888682236</v>
+        <v>0.943539925247452</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.1885551822924716</v>
+        <v>-0.7596206367931251</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.1411560352501725</v>
+        <v>0.1337117508352408</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5140902393882557</v>
+        <v>-0.07403020857614677</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.00124645458198128</v>
+        <v>0.1153815181970236</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02293024047162344</v>
+        <v>0.4293041542414215</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.167952585268016</v>
+        <v>-0.1401563555171501</v>
       </c>
       <c r="J11" t="n">
-        <v>0.08469848884430112</v>
+        <v>0.008429939735171232</v>
       </c>
       <c r="K11" t="n">
-        <v>0.006531560191316547</v>
+        <v>0.06156697036107306</v>
       </c>
       <c r="L11" t="n">
-        <v>0.01012275231118172</v>
+        <v>-0.2076567611287644</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-0.00720015067614148</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.07031489109538705</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-0.01464475322703016</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.01230576607415479</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-0.005229162616819596</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-1.218249057114873e-17</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-6.956076262717698e-19</v>
       </c>
     </row>
     <row r="12">
@@ -1611,73 +2661,115 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.3930794990060364</v>
+        <v>-0.3128864053420523</v>
       </c>
       <c r="C12" t="n">
-        <v>1.13865226421693</v>
+        <v>0.9227405557195976</v>
       </c>
       <c r="D12" t="n">
-        <v>-1.499934813156435</v>
+        <v>1.556651528663652</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1038917388659296</v>
+        <v>-1.128543476568866</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3303547473777391</v>
+        <v>-0.4327450082313611</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.09484114557959519</v>
+        <v>0.04346658778523278</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.3248751749096153</v>
+        <v>0.4268265345368618</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.1565109880937127</v>
+        <v>0.4496948743444826</v>
       </c>
       <c r="J12" t="n">
-        <v>0.04159834705758544</v>
+        <v>-0.07253297166681713</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.004352556418899105</v>
+        <v>0.1902954231980766</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.01687876480850359</v>
+        <v>-0.07286333633669674</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-0.09162267112490832</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-0.04240768912729317</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.04309593376409152</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.002006029613941106</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.0001212533674676183</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-1.137625440373282e-17</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-3.987373176412628e-19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>-1.001180799576471</v>
+        <v>-1.317579605158018</v>
       </c>
       <c r="C13" t="n">
-        <v>0.004526488647274396</v>
+        <v>1.018372997503429</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.5167039182971834</v>
+        <v>-0.4306020589299386</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.5092150947048052</v>
+        <v>-0.133572613858968</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2584201206651027</v>
+        <v>-0.225734416804669</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.01034181459199156</v>
+        <v>0.1883921174227255</v>
       </c>
       <c r="H13" t="n">
-        <v>0.03187105467832782</v>
+        <v>-0.01389278880086208</v>
       </c>
       <c r="I13" t="n">
-        <v>0.101157913146768</v>
+        <v>0.2324135206389323</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.04677486169473474</v>
+        <v>-0.1769549848720554</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03141669801518642</v>
+        <v>-0.1729075393725435</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.01265993121666253</v>
+        <v>0.02033892518580979</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.02299916297882027</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-0.01864284426739579</v>
+      </c>
+      <c r="O13" t="n">
+        <v>-0.01780875299812209</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.0123805231538932</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>-0.009774614881993786</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-5.211120618197549e-17</v>
+      </c>
+      <c r="S13" t="n">
+        <v>2.490307525445208e-18</v>
       </c>
     </row>
     <row r="14">
@@ -1687,73 +2779,115 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-1.594132921442637</v>
+        <v>-2.062348374473352</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.3476895016718284</v>
+        <v>1.066563327733697</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1710043614234952</v>
+        <v>-1.024143666791429</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1995837348905727</v>
+        <v>0.2609243208506203</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2901838727391026</v>
+        <v>-0.2319575803460575</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.03302516042291687</v>
+        <v>-0.2456325632163362</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1139580726504399</v>
+        <v>0.3389663788635657</v>
       </c>
       <c r="I14" t="n">
-        <v>0.01466665171961654</v>
+        <v>-0.2460908632812842</v>
       </c>
       <c r="J14" t="n">
-        <v>0.02585817000003613</v>
+        <v>-0.01463529608779982</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.007679230838305178</v>
+        <v>-0.002566779960753053</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.01602175122239768</v>
+        <v>-0.03074421410786141</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.1503666470835425</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-0.02353399811444229</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.0448335754209867</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.01954193686681036</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.01095284342027528</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-4.1435362124519e-17</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-1.522737217618912e-18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>-1.812859114950376</v>
+        <v>-2.422319616999643</v>
       </c>
       <c r="C15" t="n">
-        <v>-1.058147112763505</v>
+        <v>-0.2190987326891655</v>
       </c>
       <c r="D15" t="n">
-        <v>0.315377654848098</v>
+        <v>-1.536762529986881</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.08278789713652765</v>
+        <v>0.4125093178086977</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.202153096702059</v>
+        <v>-0.2789059679901754</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.118059937043984</v>
+        <v>-0.6638310155721727</v>
       </c>
       <c r="H15" t="n">
-        <v>0.006109183673144088</v>
+        <v>0.08335892048832241</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.05647762767469818</v>
+        <v>-0.1420080619641978</v>
       </c>
       <c r="J15" t="n">
-        <v>0.03231403668466764</v>
+        <v>0.005059398902696044</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.04835591582396101</v>
+        <v>0.04849915615776804</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.009112653354603163</v>
+        <v>-0.06344696436343461</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.01016433669440362</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.001635326562541076</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.01300783150569474</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-0.04368035719795745</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-0.006680966502189327</v>
+      </c>
+      <c r="R15" t="n">
+        <v>-5.012772950897007e-17</v>
+      </c>
+      <c r="S15" t="n">
+        <v>2.402602164366244e-18</v>
       </c>
     </row>
     <row r="16">
@@ -1763,37 +2897,58 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.8888461732917488</v>
+        <v>-1.225357113024292</v>
       </c>
       <c r="C16" t="n">
-        <v>0.07781821200570219</v>
+        <v>1.006842160552219</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.5917516134974592</v>
+        <v>-0.3477149551900535</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1243937890814983</v>
+        <v>-0.2755591390641861</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1265457564087747</v>
+        <v>0.04521877247819586</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0152378268373352</v>
+        <v>-0.04663886153584561</v>
       </c>
       <c r="H16" t="n">
-        <v>0.02607449167463132</v>
+        <v>-0.01508841182740166</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08571189752776685</v>
+        <v>0.1098600077343457</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.02675951365607826</v>
+        <v>-0.1014345272179989</v>
       </c>
       <c r="K16" t="n">
-        <v>0.006524548672384621</v>
+        <v>-0.1211854574480216</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.01428688610912774</v>
+        <v>0.04136514836972682</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-0.01407382958812328</v>
+      </c>
+      <c r="N16" t="n">
+        <v>-0.03477117288077908</v>
+      </c>
+      <c r="O16" t="n">
+        <v>-0.006077976004108659</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.00957145280266815</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-0.01086709694831974</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-4.027300729140997e-17</v>
+      </c>
+      <c r="S16" t="n">
+        <v>-4.054297156610868e-18</v>
       </c>
     </row>
     <row r="17">
@@ -1803,37 +2958,58 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-1.524628609196013</v>
+        <v>-1.936872763126338</v>
       </c>
       <c r="C17" t="n">
-        <v>0.95267971488147</v>
+        <v>0.3295468679414648</v>
       </c>
       <c r="D17" t="n">
-        <v>1.64304909257073</v>
+        <v>0.1057519562195742</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.1485685106500888</v>
+        <v>2.020224441339073</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1820296746226336</v>
+        <v>0.5005080496119498</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.1972767447624894</v>
+        <v>-0.1539972624210404</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.01581729945930283</v>
+        <v>0.03898210869068159</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0464267746613047</v>
+        <v>0.08793137429068874</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.04749493243565358</v>
+        <v>-0.07115618035507396</v>
       </c>
       <c r="K17" t="n">
-        <v>0.01030071348477006</v>
+        <v>0.02845903209685407</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.004874146905594972</v>
+        <v>0.007508692466188809</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.1025453605113609</v>
+      </c>
+      <c r="N17" t="n">
+        <v>-0.03047335432715342</v>
+      </c>
+      <c r="O17" t="n">
+        <v>-0.02460856361577184</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-0.003514772611255284</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.005156639203020045</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-4.103936233986979e-17</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-1.684879061545644e-19</v>
       </c>
     </row>
     <row r="18">
@@ -1843,37 +3019,58 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.194543536507407</v>
+        <v>2.578184289753111</v>
       </c>
       <c r="C18" t="n">
-        <v>1.38548372626067</v>
+        <v>2.073030557367749</v>
       </c>
       <c r="D18" t="n">
-        <v>-1.976773392341549</v>
+        <v>1.234524428636279</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.03886710478072273</v>
+        <v>-1.258182289057655</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.5174550263107826</v>
+        <v>-0.4061928291566426</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.1907489904535163</v>
+        <v>-0.6795344076936661</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0971829066543082</v>
+        <v>-0.3019107253623303</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.01265414674352174</v>
+        <v>0.02876876175262505</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.01558821973023284</v>
+        <v>0.1447194981741752</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.006264190181606877</v>
+        <v>-0.02346959933866152</v>
       </c>
       <c r="L18" t="n">
-        <v>0.005704802869027132</v>
+        <v>0.00927521866568781</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.02658645860950509</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.01043956838152001</v>
+      </c>
+      <c r="O18" t="n">
+        <v>-0.006231154752540411</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-0.004556857599913921</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.001852498389093641</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-2.971051184751426e-17</v>
+      </c>
+      <c r="S18" t="n">
+        <v>4.27974603258717e-18</v>
       </c>
     </row>
     <row r="19">
@@ -1883,37 +3080,58 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-1.691944996850117</v>
+        <v>-2.045528996678056</v>
       </c>
       <c r="C19" t="n">
-        <v>-1.292068371420996</v>
+        <v>-1.702823965670773</v>
       </c>
       <c r="D19" t="n">
-        <v>0.5378610291288173</v>
+        <v>-0.7065201410182897</v>
       </c>
       <c r="E19" t="n">
-        <v>0.09869372079323448</v>
+        <v>-0.2786197923253201</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2143415522111472</v>
+        <v>0.3391855124865656</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.06498058858893137</v>
+        <v>0.5847275412116277</v>
       </c>
       <c r="H19" t="n">
-        <v>0.033800034062642</v>
+        <v>-0.5401288664024988</v>
       </c>
       <c r="I19" t="n">
-        <v>0.02275133366496494</v>
+        <v>0.2511258301870062</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.002825767628980197</v>
+        <v>0.07775043764950741</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0005395987936683424</v>
+        <v>-0.04398459496908277</v>
       </c>
       <c r="L19" t="n">
-        <v>0.001433864886508726</v>
+        <v>0.01536277103139732</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-0.0154333848964265</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.0134565647623171</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.02728834051835376</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.004599769238879711</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.01001143423801158</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-6.706451582633748e-17</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-1.271925805364323e-18</v>
       </c>
     </row>
     <row r="20">
@@ -1923,37 +3141,58 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-1.599153871121226</v>
+        <v>-1.888440434176897</v>
       </c>
       <c r="C20" t="n">
-        <v>-1.212990222011216</v>
+        <v>-1.28566382924301</v>
       </c>
       <c r="D20" t="n">
-        <v>0.3785567862294375</v>
+        <v>-1.007311257065743</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.163916779867121</v>
+        <v>0.1507429120969501</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.3996525756127634</v>
+        <v>-0.6260598185892906</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.177067662649676</v>
+        <v>-0.3537326145183517</v>
       </c>
       <c r="H20" t="n">
-        <v>0.028458598520793</v>
+        <v>-0.07633457164120434</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.0221556721124623</v>
+        <v>-0.06985638047757212</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.03434799975310081</v>
+        <v>0.3428272283278891</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.007489337622519068</v>
+        <v>0.129758643252488</v>
       </c>
       <c r="L20" t="n">
-        <v>0.002579306398764239</v>
+        <v>0.1502555980541071</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.0106387515922173</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-0.007799939678218976</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.01268941385363708</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.01666866453731865</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>-0.006608152424999049</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-7.133567673349404e-18</v>
+      </c>
+      <c r="S20" t="n">
+        <v>-1.013259426819103e-19</v>
       </c>
     </row>
     <row r="21">
@@ -1963,37 +3202,58 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-1.84854832205883</v>
+        <v>-2.151018865687908</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.3757978099476215</v>
+        <v>-0.4988642226899411</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.19138002592106</v>
+        <v>-0.07258815228989327</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0554476882912146</v>
+        <v>-0.2886674268942079</v>
       </c>
       <c r="F21" t="n">
-        <v>0.1374992996792788</v>
+        <v>-0.3209824025903138</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.08318172823576797</v>
+        <v>0.02472541931235114</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1048580378284781</v>
+        <v>0.2443792983783982</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.03636228963942246</v>
+        <v>0.1583901276388961</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.04481042946923812</v>
+        <v>0.06777751961747755</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.01843592136868442</v>
+        <v>0.1012648098911471</v>
       </c>
       <c r="L21" t="n">
-        <v>0.00953060720494343</v>
+        <v>0.05912708757144384</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.01482057103286565</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.0162489895374485</v>
+      </c>
+      <c r="O21" t="n">
+        <v>3.116106818556708e-05</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.007762797537497854</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.005619337405225027</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-2.546261110579915e-17</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-2.846772172050219e-20</v>
       </c>
     </row>
     <row r="22">
@@ -2003,37 +3263,58 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-1.776383893066511</v>
+        <v>-2.075268270034464</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.4739314405670856</v>
+        <v>0.04815669840461035</v>
       </c>
       <c r="D22" t="n">
-        <v>0.01300906940912093</v>
+        <v>-0.5575467248998303</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.01998207311831292</v>
+        <v>-0.0614661856459592</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4712706375015944</v>
+        <v>0.1465792028800021</v>
       </c>
       <c r="G22" t="n">
-        <v>0.03853303619735059</v>
+        <v>0.4951902517974857</v>
       </c>
       <c r="H22" t="n">
-        <v>0.09621593812606465</v>
+        <v>0.2165891167583675</v>
       </c>
       <c r="I22" t="n">
-        <v>0.02136370329664621</v>
+        <v>0.02096850914800794</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.0177595515801304</v>
+        <v>0.08882592621745247</v>
       </c>
       <c r="K22" t="n">
-        <v>0.009648052229159409</v>
+        <v>-0.07433725108836706</v>
       </c>
       <c r="L22" t="n">
-        <v>0.01052459786761701</v>
+        <v>0.04491725710817637</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.004382194350270866</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.05935243378614505</v>
+      </c>
+      <c r="O22" t="n">
+        <v>-0.003250227329878335</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.02367754633685587</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>-0.006572213731882622</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-6.758028685895034e-19</v>
+      </c>
+      <c r="S22" t="n">
+        <v>4.071871348395613e-19</v>
       </c>
     </row>
     <row r="23">
@@ -2043,37 +3324,58 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.5597942230702402</v>
+        <v>-0.6920766353228729</v>
       </c>
       <c r="C23" t="n">
-        <v>0.1882949896369955</v>
+        <v>-0.1023951958760968</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6016558962295069</v>
+        <v>0.1008114433108298</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.48119487015334</v>
+        <v>0.6978795101150544</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.5163500788164189</v>
+        <v>-0.3288297790725573</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1103003899082767</v>
+        <v>-0.1719697134081303</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.2574071582107112</v>
+        <v>-0.5515641227008</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1699382685127831</v>
+        <v>0.006661777691369552</v>
       </c>
       <c r="J23" t="n">
-        <v>0.04079875473019842</v>
+        <v>-0.2792816035815391</v>
       </c>
       <c r="K23" t="n">
-        <v>0.01888209832234048</v>
+        <v>0.2278917109692917</v>
       </c>
       <c r="L23" t="n">
-        <v>0.008878976645610982</v>
+        <v>0.05503764413241971</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-0.01226804313695881</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.05707599182516761</v>
+      </c>
+      <c r="O23" t="n">
+        <v>-0.02408810311263115</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.02181863970948184</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>-0.009634849795917428</v>
+      </c>
+      <c r="R23" t="n">
+        <v>-2.691914956213542e-17</v>
+      </c>
+      <c r="S23" t="n">
+        <v>-2.373883638667052e-19</v>
       </c>
     </row>
     <row r="24">
@@ -2083,37 +3385,58 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.188614378948753</v>
+        <v>2.589475945579051</v>
       </c>
       <c r="C24" t="n">
-        <v>1.429814662901902</v>
+        <v>2.09833772972532</v>
       </c>
       <c r="D24" t="n">
-        <v>-1.98890761918643</v>
+        <v>1.263664313004268</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.02218777904216162</v>
+        <v>-1.251679922002106</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.4450594681114973</v>
+        <v>-0.3862976701886664</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.1583388302148715</v>
+        <v>-0.6540960885318298</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1181678268367057</v>
+        <v>-0.2323476460832037</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.0278469540987407</v>
+        <v>0.02743614435302434</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.02416264098507272</v>
+        <v>0.1484711336825026</v>
       </c>
       <c r="K24" t="n">
-        <v>-0.001516259597413297</v>
+        <v>-0.06236480892200093</v>
       </c>
       <c r="L24" t="n">
-        <v>0.02394111815727526</v>
+        <v>-0.001200674287883041</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-0.001020741715475788</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.04281498440343133</v>
+      </c>
+      <c r="O24" t="n">
+        <v>-0.03103257172660757</v>
+      </c>
+      <c r="P24" t="n">
+        <v>-0.004967109515933287</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.005802222325037061</v>
+      </c>
+      <c r="R24" t="n">
+        <v>-2.576258879216532e-17</v>
+      </c>
+      <c r="S24" t="n">
+        <v>-3.874159173612116e-18</v>
       </c>
     </row>
     <row r="25">
@@ -2123,37 +3446,58 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-1.588176757884407</v>
+        <v>-2.051504884962058</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.339893523328794</v>
+        <v>0.468942013981481</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.1868244476217634</v>
+        <v>-0.7942807094054373</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.09778182043690695</v>
+        <v>0.07119428355215227</v>
       </c>
       <c r="F25" t="n">
-        <v>0.2344612145171157</v>
+        <v>-0.0867049975407274</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.03075961694488372</v>
+        <v>-0.1886628213347447</v>
       </c>
       <c r="H25" t="n">
-        <v>0.1018677464829768</v>
+        <v>0.2566702219406772</v>
       </c>
       <c r="I25" t="n">
-        <v>0.01675825163002015</v>
+        <v>0.03754941178236344</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.02375215527575084</v>
+        <v>0.02696648064898327</v>
       </c>
       <c r="K25" t="n">
-        <v>0.006950933992989713</v>
+        <v>-0.1357450359558077</v>
       </c>
       <c r="L25" t="n">
-        <v>-0.006097904691384199</v>
+        <v>0.0308156230905021</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.007801400621507075</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-0.01179895192337467</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.004921331427073626</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.009394897851817798</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>-0.006809346380130813</v>
+      </c>
+      <c r="R25" t="n">
+        <v>5.484060317501741e-17</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1.749229402186149e-21</v>
       </c>
     </row>
     <row r="26">
@@ -2163,37 +3507,58 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.8668350123925005</v>
+        <v>-0.8304172298501795</v>
       </c>
       <c r="C26" t="n">
-        <v>0.2223404801442957</v>
+        <v>1.129109567550707</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.4358408789773653</v>
+        <v>0.01005398239303134</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1773503386380494</v>
+        <v>-0.335119161042685</v>
       </c>
       <c r="F26" t="n">
-        <v>1.019502115479428</v>
+        <v>0.5402432082518132</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1654574101445727</v>
+        <v>1.028985621266393</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.01076908647392176</v>
+        <v>0.5253836118691168</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.01797278777000173</v>
+        <v>-0.0572713752830917</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.03634910718194219</v>
+        <v>0.1169399772567543</v>
       </c>
       <c r="K26" t="n">
-        <v>0.02283067523638826</v>
+        <v>0.03988951428027422</v>
       </c>
       <c r="L26" t="n">
-        <v>0.02028019805164913</v>
+        <v>0.06389085584966039</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-0.05161952489976897</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-0.02176433731152434</v>
+      </c>
+      <c r="O26" t="n">
+        <v>-0.04631029326925369</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.002738139778784836</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.007293940658989986</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-4.42271182767766e-17</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.927717117882199e-18</v>
       </c>
     </row>
     <row r="27">
@@ -2203,37 +3568,58 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6.337189904968314</v>
+        <v>8.361279828529446</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.1216064724641592</v>
+        <v>-1.422545697026402</v>
       </c>
       <c r="D27" t="n">
-        <v>0.8272937400916386</v>
+        <v>0.5968836794854684</v>
       </c>
       <c r="E27" t="n">
-        <v>-2.512326712223067</v>
+        <v>1.232750979143935</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.1529435912778404</v>
+        <v>-3.124441298239125</v>
       </c>
       <c r="G27" t="n">
-        <v>0.3692318088745061</v>
+        <v>0.5121895434002083</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.02228879231628399</v>
+        <v>0.1766176504222506</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.0893156002422088</v>
+        <v>-0.03222894038872992</v>
       </c>
       <c r="J27" t="n">
-        <v>-0.05142027785367383</v>
+        <v>-0.02750154976802619</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.01138809159956398</v>
+        <v>-0.05832328221831883</v>
       </c>
       <c r="L27" t="n">
-        <v>0.001554517662881983</v>
+        <v>-0.006726024464907595</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.01000694911742162</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.002347730252918863</v>
+      </c>
+      <c r="O27" t="n">
+        <v>-0.002312726790429185</v>
+      </c>
+      <c r="P27" t="n">
+        <v>-0.007416303764439141</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.001820250971962841</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-1.858339463974031e-17</v>
+      </c>
+      <c r="S27" t="n">
+        <v>-1.527123495979347e-19</v>
       </c>
     </row>
     <row r="28">
@@ -2243,37 +3629,58 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-0.08718793964779278</v>
+        <v>0.1092670670872819</v>
       </c>
       <c r="C28" t="n">
-        <v>-0.1889905664547802</v>
+        <v>-2.285149125796217</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.3491096822733129</v>
+        <v>1.713003788963565</v>
       </c>
       <c r="E28" t="n">
-        <v>1.268053297941188</v>
+        <v>-1.582609562797971</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.4706557477228569</v>
+        <v>0.4749191412927455</v>
       </c>
       <c r="G28" t="n">
-        <v>0.395319895474659</v>
+        <v>0.03112864819013988</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.04854137038544658</v>
+        <v>-0.03681323419959542</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.01418823307251272</v>
+        <v>-0.3092160975177564</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.0233787443145742</v>
+        <v>-0.1353276722643036</v>
       </c>
       <c r="K28" t="n">
-        <v>0.02324295801132854</v>
+        <v>0.02282465233687208</v>
       </c>
       <c r="L28" t="n">
-        <v>0.006910913263670514</v>
+        <v>-0.04037312255667153</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.0519752181675476</v>
+      </c>
+      <c r="N28" t="n">
+        <v>-0.008580970544088283</v>
+      </c>
+      <c r="O28" t="n">
+        <v>-0.03105852388621247</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.01228452733607002</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.01117389787848671</v>
+      </c>
+      <c r="R28" t="n">
+        <v>-3.422874941481027e-18</v>
+      </c>
+      <c r="S28" t="n">
+        <v>2.103266408908863e-19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
3D PCA plots, increased n trials, descriptions
</commit_message>
<xml_diff>
--- a/api_pca_results.xlsx
+++ b/api_pca_results.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,13 +448,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6829876176034376</v>
+        <v>0.6871068153976634</v>
       </c>
       <c r="C2" t="n">
-        <v>68.29876176034377</v>
+        <v>68.71068153976634</v>
       </c>
       <c r="D2" t="n">
-        <v>68.29876176034377</v>
+        <v>68.71068153976634</v>
       </c>
     </row>
     <row r="3">
@@ -464,13 +464,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1021743313291748</v>
+        <v>0.1147039659334233</v>
       </c>
       <c r="C3" t="n">
-        <v>10.21743313291748</v>
+        <v>11.47039659334233</v>
       </c>
       <c r="D3" t="n">
-        <v>78.51619489326124</v>
+        <v>80.18107813310866</v>
       </c>
     </row>
     <row r="4">
@@ -480,13 +480,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.09965817367375222</v>
+        <v>0.08639986712014874</v>
       </c>
       <c r="C4" t="n">
-        <v>9.965817367375223</v>
+        <v>8.639986712014874</v>
       </c>
       <c r="D4" t="n">
-        <v>88.48201226063645</v>
+        <v>88.82106484512353</v>
       </c>
     </row>
     <row r="5">
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05347396723869859</v>
+        <v>0.04983761540690027</v>
       </c>
       <c r="C5" t="n">
-        <v>5.347396723869859</v>
+        <v>4.983761540690026</v>
       </c>
       <c r="D5" t="n">
-        <v>93.82940898450632</v>
+        <v>93.80482638581356</v>
       </c>
     </row>
     <row r="6">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.03989212465983037</v>
+        <v>0.0380128481545902</v>
       </c>
       <c r="C6" t="n">
-        <v>3.989212465983037</v>
+        <v>3.80128481545902</v>
       </c>
       <c r="D6" t="n">
-        <v>97.81862145048935</v>
+        <v>97.60611120127257</v>
       </c>
     </row>
     <row r="7">
@@ -528,13 +528,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01171960059564808</v>
+        <v>0.01276992063150958</v>
       </c>
       <c r="C7" t="n">
-        <v>1.171960059564808</v>
+        <v>1.276992063150959</v>
       </c>
       <c r="D7" t="n">
-        <v>98.99058151005416</v>
+        <v>98.88310326442354</v>
       </c>
     </row>
     <row r="8">
@@ -544,13 +544,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.005749016023262258</v>
+        <v>0.005631170175228433</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5749016023262259</v>
+        <v>0.5631170175228433</v>
       </c>
       <c r="D8" t="n">
-        <v>99.56548311238038</v>
+        <v>99.44622028194637</v>
       </c>
     </row>
     <row r="9">
@@ -560,13 +560,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.002160218363405858</v>
+        <v>0.002989059878532225</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2160218363405858</v>
+        <v>0.2989059878532225</v>
       </c>
       <c r="D9" t="n">
-        <v>99.78150494872096</v>
+        <v>99.7451262697996</v>
       </c>
     </row>
     <row r="10">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0009948917211693689</v>
+        <v>0.001176661545088224</v>
       </c>
       <c r="C10" t="n">
-        <v>0.09948917211693689</v>
+        <v>0.1176661545088224</v>
       </c>
       <c r="D10" t="n">
-        <v>99.88099412083791</v>
+        <v>99.86279242430842</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0005113746506266259</v>
+        <v>0.0006762264681849886</v>
       </c>
       <c r="C11" t="n">
-        <v>0.05113746506266259</v>
+        <v>0.06762264681849886</v>
       </c>
       <c r="D11" t="n">
-        <v>99.93213158590058</v>
+        <v>99.93041507112692</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.000306998414899189</v>
+        <v>0.0002879053113380409</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0306998414899189</v>
+        <v>0.02879053113380409</v>
       </c>
       <c r="D12" t="n">
-        <v>99.9628314273905</v>
+        <v>99.95920560226072</v>
       </c>
     </row>
     <row r="13">
@@ -624,13 +624,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0002347067736501655</v>
+        <v>0.0002394061008127609</v>
       </c>
       <c r="C13" t="n">
-        <v>0.02347067736501655</v>
+        <v>0.02394061008127609</v>
       </c>
       <c r="D13" t="n">
-        <v>99.98630210475551</v>
+        <v>99.98314621234201</v>
       </c>
     </row>
     <row r="14">
@@ -640,13 +640,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8.031444037406305e-05</v>
+        <v>8.921917640128673e-05</v>
       </c>
       <c r="C14" t="n">
-        <v>0.008031444037406306</v>
+        <v>0.008921917640128672</v>
       </c>
       <c r="D14" t="n">
-        <v>99.99433354879291</v>
+        <v>99.99206812998213</v>
       </c>
     </row>
     <row r="15">
@@ -656,13 +656,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.51076004710023e-05</v>
+        <v>4.517446710136991e-05</v>
       </c>
       <c r="C15" t="n">
-        <v>0.003510760047100229</v>
+        <v>0.004517446710136991</v>
       </c>
       <c r="D15" t="n">
-        <v>99.99784430884002</v>
+        <v>99.99658557669227</v>
       </c>
     </row>
     <row r="16">
@@ -672,13 +672,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.813830806432101e-05</v>
+        <v>2.511615780027677e-05</v>
       </c>
       <c r="C16" t="n">
-        <v>0.001813830806432101</v>
+        <v>0.002511615780027677</v>
       </c>
       <c r="D16" t="n">
-        <v>99.99965813964644</v>
+        <v>99.99909719247229</v>
       </c>
     </row>
     <row r="17">
@@ -688,13 +688,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.418603535405527e-06</v>
+        <v>6.325853751211017e-06</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0003418603535405527</v>
+        <v>0.0006325853751211018</v>
       </c>
       <c r="D17" t="n">
-        <v>99.99999999999997</v>
+        <v>99.99972977784742</v>
       </c>
     </row>
     <row r="18">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6.098902137787327e-35</v>
+        <v>2.64599872795949e-06</v>
       </c>
       <c r="C18" t="n">
-        <v>6.098902137787327e-33</v>
+        <v>0.000264599872795949</v>
       </c>
       <c r="D18" t="n">
-        <v>99.99999999999997</v>
+        <v>99.99999437772023</v>
       </c>
     </row>
     <row r="19">
@@ -720,13 +720,61 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.651066957992938e-37</v>
+        <v>5.622279776542175e-08</v>
       </c>
       <c r="C19" t="n">
-        <v>1.651066957992938e-35</v>
+        <v>5.622279776542175e-06</v>
       </c>
       <c r="D19" t="n">
-        <v>99.99999999999997</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PC19</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3.010004269667515e-34</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3.010004269667515e-32</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PC20</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2.277489222979388e-35</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2.277489222979388e-33</v>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PC21</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.105990246001376e-38</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.105990246001376e-36</v>
+      </c>
+      <c r="D22" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -740,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -834,6 +882,21 @@
           <t>PC18</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>PC19</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>PC20</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>PC21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -842,58 +905,67 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.292555911505707</v>
+        <v>0.268956248608727</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01209496908042476</v>
+        <v>-0.0181667812065519</v>
       </c>
       <c r="D2" t="n">
-        <v>0.006114071157475818</v>
+        <v>0.01146312897235018</v>
       </c>
       <c r="E2" t="n">
-        <v>0.05021254613209371</v>
+        <v>0.04808782237399527</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.002679372930503698</v>
+        <v>-0.009676420011449183</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05083684903521189</v>
+        <v>0.04511054891420666</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1563538441034655</v>
+        <v>0.1104035852541935</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.005121518871821546</v>
+        <v>-0.01551459363645136</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.08670351957530033</v>
+        <v>-0.1050240651624335</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.1149450627430896</v>
+        <v>0.02259608581984881</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.2066868790709916</v>
+        <v>-0.09090452873814527</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.2004029363581004</v>
+        <v>-0.2409230100461537</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.03183958071116434</v>
+        <v>0.05258967244336366</v>
       </c>
       <c r="O2" t="n">
-        <v>-0.2734289408792462</v>
+        <v>-0.118895098278593</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.2278569511049212</v>
+        <v>-0.2176717104549385</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.8082914972436338</v>
+        <v>0.0243601160962445</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>0.7234896836083495</v>
       </c>
       <c r="S2" t="n">
-        <v>-0</v>
+        <v>-0.4941344117110554</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1.389453533374389e-14</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1.408982813608102e-14</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-7.530685385615085e-17</v>
       </c>
     </row>
     <row r="3">
@@ -903,58 +975,67 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.2241232219669497</v>
+        <v>-0.2010626868704874</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2667638534404871</v>
+        <v>0.3159407588276705</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3430698658226735</v>
+        <v>0.1680229640479637</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01026657043827786</v>
+        <v>0.2046043485843562</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2375212462789646</v>
+        <v>0.2949706380354891</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2276669810117067</v>
+        <v>0.225039697326381</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6678380905262079</v>
+        <v>0.6049500030954974</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02869388608615136</v>
+        <v>-0.1818973476668581</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1185639113567169</v>
+        <v>-0.1436365277818083</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.3539327146075258</v>
+        <v>0.3690956062930764</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1238665999499238</v>
+        <v>0.2165683575919894</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.06574464320072705</v>
+        <v>-0.0626013698620851</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1607521972011305</v>
+        <v>0.1735845584317646</v>
       </c>
       <c r="O3" t="n">
-        <v>0.009907394569537209</v>
+        <v>0.03866114665031283</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1378435832993911</v>
+        <v>0.1103769965626532</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.04233795658632378</v>
+        <v>-0.01518366379139055</v>
       </c>
       <c r="R3" t="n">
-        <v>-8.467780417813657e-17</v>
+        <v>-0.03471954325551194</v>
       </c>
       <c r="S3" t="n">
-        <v>8.053890807863828e-18</v>
+        <v>0.005452003319947968</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-4.238743202471189e-16</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-4.766567083553054e-16</v>
+      </c>
+      <c r="V3" t="n">
+        <v>6.524108837867958e-18</v>
       </c>
     </row>
     <row r="4">
@@ -964,58 +1045,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2722901440003537</v>
+        <v>0.2479018316868928</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.05957395279525762</v>
+        <v>-0.2207104505175368</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1969698134079306</v>
+        <v>0.000183496148284981</v>
       </c>
       <c r="E4" t="n">
-        <v>0.07208109221823868</v>
+        <v>0.06109984029723119</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2411553208873852</v>
+        <v>0.1402070591777874</v>
       </c>
       <c r="G4" t="n">
-        <v>0.09588486732070536</v>
+        <v>-0.05584105048542694</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3469222669147973</v>
+        <v>0.2839494133380221</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3635630111396347</v>
+        <v>-0.4000447933280219</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.2647077290243893</v>
+        <v>0.08635512478964161</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5561124727170722</v>
+        <v>-0.5489155261862945</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3243537849565395</v>
+        <v>0.2015807435937957</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2276205532438263</v>
+        <v>0.4696701418947953</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1015348738657216</v>
+        <v>0.1847625698366081</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.07197467541228712</v>
+        <v>-0.08405886910746908</v>
       </c>
       <c r="P4" t="n">
-        <v>0.07841652423921809</v>
+        <v>0.06085293742015362</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.02113569206015313</v>
+        <v>-0.06431974585082423</v>
       </c>
       <c r="R4" t="n">
-        <v>1.443913504521839e-16</v>
+        <v>0.05997430194740221</v>
       </c>
       <c r="S4" t="n">
-        <v>6.150081859228522e-18</v>
+        <v>0.005345861441847274</v>
+      </c>
+      <c r="T4" t="n">
+        <v>3.98835802394221e-16</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-8.703558938045386e-16</v>
+      </c>
+      <c r="V4" t="n">
+        <v>2.760163193636611e-18</v>
       </c>
     </row>
     <row r="5">
@@ -1025,58 +1115,67 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.2898054787715753</v>
+        <v>0.266800466412665</v>
       </c>
       <c r="C5" t="n">
-        <v>0.04756100127849142</v>
+        <v>0.03971188334951097</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06205077496719423</v>
+        <v>0.02661887811782359</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0254066456542625</v>
+        <v>0.02869500092733667</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.06115884665335814</v>
+        <v>-0.03213891353281046</v>
       </c>
       <c r="G5" t="n">
-        <v>0.007601193255699588</v>
+        <v>0.05577110876676021</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1189238812550072</v>
+        <v>-0.1602292216737478</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.2261060331339345</v>
+        <v>0.2052230114322793</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.531871899860854</v>
+        <v>-0.4930873470462018</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.3730571799596994</v>
+        <v>-0.1353365593806349</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6030011046023132</v>
+        <v>0.7259824019661635</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.1340860837545559</v>
+        <v>-0.1214038448599796</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.1235729227257736</v>
+        <v>-0.1902751645190702</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1278686198975868</v>
+        <v>0.09735963115364847</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.04807386741652576</v>
+        <v>0.03071680293654122</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.05108222387023936</v>
+        <v>-0.003975287408027954</v>
       </c>
       <c r="R5" t="n">
-        <v>4.049624119736836e-17</v>
+        <v>-0.06119846204884539</v>
       </c>
       <c r="S5" t="n">
-        <v>-6.835317499249891e-18</v>
+        <v>-0.01211301623889445</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-2.522722670784289e-16</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-1.753309186016848e-16</v>
+      </c>
+      <c r="V5" t="n">
+        <v>8.007415431288299e-18</v>
       </c>
     </row>
     <row r="6">
@@ -1086,58 +1185,67 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2876214665551332</v>
+        <v>0.2621372488160316</v>
       </c>
       <c r="C6" t="n">
-        <v>0.001787972518615037</v>
+        <v>-0.1336467827723347</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1366140040501975</v>
+        <v>0.03446413757496276</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01167532492100639</v>
+        <v>-0.03159197838646451</v>
       </c>
       <c r="F6" t="n">
-        <v>0.03294395993648866</v>
+        <v>0.003668566977272201</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.05965352134817738</v>
+        <v>-0.08879121682439223</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.06907502934928669</v>
+        <v>-0.139003700738126</v>
       </c>
       <c r="I6" t="n">
-        <v>0.135078059703383</v>
+        <v>-0.1144381615610531</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3064766457749984</v>
+        <v>-0.0937240930451488</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.4319076220979891</v>
+        <v>0.5977476234439737</v>
       </c>
       <c r="L6" t="n">
-        <v>0.09769264231103399</v>
+        <v>0.02657864341838535</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6700097985733899</v>
+        <v>0.5640310645122193</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2431406035452383</v>
+        <v>-0.04323829294546511</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.0003113062376722247</v>
+        <v>0.2978995863686603</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.2695498369770317</v>
+        <v>-0.2770653151490249</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.01029714629289662</v>
+        <v>-0.1226282868489727</v>
       </c>
       <c r="R6" t="n">
-        <v>6.630346260352756e-17</v>
+        <v>0.05969468302377673</v>
       </c>
       <c r="S6" t="n">
-        <v>5.386808643152657e-20</v>
+        <v>0.004166877692738113</v>
+      </c>
+      <c r="T6" t="n">
+        <v>1.614397268044125e-16</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-5.186779473313324e-16</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3.573699266105726e-17</v>
       </c>
     </row>
     <row r="7">
@@ -1147,58 +1255,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2925300997828106</v>
+        <v>0.2689018855020133</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01230617664597992</v>
+        <v>-0.02109358149891201</v>
       </c>
       <c r="D7" t="n">
-        <v>0.003162235340474906</v>
+        <v>0.01253076280834873</v>
       </c>
       <c r="E7" t="n">
-        <v>0.04364090383615486</v>
+        <v>0.04587546970958114</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01760419526273376</v>
+        <v>0.00860399276535581</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0463947277879276</v>
+        <v>0.03251380724996265</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1721191329674826</v>
+        <v>0.1249087118507633</v>
       </c>
       <c r="I7" t="n">
-        <v>0.05992799386784303</v>
+        <v>-0.06506594776549264</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.05706901328501741</v>
+        <v>-0.07584945771070435</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.09095786880484362</v>
+        <v>0.02771380294190157</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.2773625019867743</v>
+        <v>-0.1948576153425955</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.01500630001870578</v>
+        <v>-0.11255786270284</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.3714118780495689</v>
+        <v>-0.2665807363489316</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.1531105925557019</v>
+        <v>-0.1704446136440035</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.1143650729856703</v>
+        <v>0.04023501928339557</v>
       </c>
       <c r="Q7" t="n">
-        <v>-0.3369377870260649</v>
+        <v>-0.4168969100844257</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7071067810630349</v>
+        <v>-0.2487724230658907</v>
       </c>
       <c r="S7" t="n">
-        <v>-1.321641819895752e-05</v>
+        <v>-0.09711897765140284</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.06550849419106303</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.7040293505986649</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-0.007163147663102071</v>
       </c>
     </row>
     <row r="8">
@@ -1208,58 +1325,67 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2903546916224534</v>
+        <v>0.2648464708538957</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.01771261568883749</v>
+        <v>-0.113947627093162</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.09979708694814132</v>
+        <v>0.006044560921988176</v>
       </c>
       <c r="E8" t="n">
-        <v>0.03322466957931148</v>
+        <v>0.0001036838059314202</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0343994849776547</v>
+        <v>0.005734186024948285</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.04539836251474381</v>
+        <v>-0.0645902352993806</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.08726367204004909</v>
+        <v>-0.1511862927409496</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0008027374237403433</v>
+        <v>-0.01066349397229962</v>
       </c>
       <c r="J8" t="n">
-        <v>0.03046236323845826</v>
+        <v>-0.2049680764679112</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.20284996672231</v>
+        <v>0.2727201579040633</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.1424935577357676</v>
+        <v>-0.1184976956603584</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0896259748230312</v>
+        <v>0.08991420554359626</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.03958765708207483</v>
+        <v>0.1851642905887714</v>
       </c>
       <c r="O8" t="n">
-        <v>-0.0228025381595663</v>
+        <v>-0.3526627490469761</v>
       </c>
       <c r="P8" t="n">
-        <v>0.8983632737776938</v>
+        <v>0.7161322506861563</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.117898882057618</v>
+        <v>0.2777692659667536</v>
       </c>
       <c r="R8" t="n">
-        <v>-1.8402832578503e-16</v>
+        <v>0.04746295893475298</v>
       </c>
       <c r="S8" t="n">
-        <v>2.199632688866561e-17</v>
+        <v>0.01532190652780833</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-1.098981406527453e-15</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-5.023219608664971e-16</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-6.153430831981578e-17</v>
       </c>
     </row>
     <row r="9">
@@ -1269,58 +1395,67 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2906254158479507</v>
+        <v>0.2670548536732105</v>
       </c>
       <c r="C9" t="n">
-        <v>0.09044120257993998</v>
+        <v>-0.007810914589491727</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.01392105394310344</v>
+        <v>0.0944083546817603</v>
       </c>
       <c r="E9" t="n">
-        <v>0.04903739620042843</v>
+        <v>0.04010147322431072</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.01348715058034322</v>
+        <v>-0.0242503034658413</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02352061957993946</v>
+        <v>0.00923671333885318</v>
       </c>
       <c r="H9" t="n">
-        <v>0.08535357848632902</v>
+        <v>0.06593696885287843</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1275257459639451</v>
+        <v>-0.07601234658777563</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0405877293251965</v>
+        <v>0.08500602628832447</v>
       </c>
       <c r="K9" t="n">
-        <v>0.02708399664020491</v>
+        <v>-0.1207891319118156</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.2901617295126436</v>
+        <v>-0.192916396123219</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.1585851917855154</v>
+        <v>-0.2253883947795957</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1664438188662546</v>
+        <v>-0.01316806682983661</v>
       </c>
       <c r="O9" t="n">
-        <v>0.8561907871819988</v>
+        <v>0.8085923549395622</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.08346089824307926</v>
+        <v>0.372690311001818</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.03193263451326364</v>
+        <v>0.01023920997539638</v>
       </c>
       <c r="R9" t="n">
-        <v>-6.833926941232111e-16</v>
+        <v>0.06247519695693999</v>
       </c>
       <c r="S9" t="n">
-        <v>-1.115384314749725e-17</v>
+        <v>0.02381002013156346</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-1.697432333646324e-15</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-1.255326012184096e-15</v>
+      </c>
+      <c r="V9" t="n">
+        <v>2.849008327847669e-17</v>
       </c>
     </row>
     <row r="10">
@@ -1330,58 +1465,67 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2113393296861263</v>
+        <v>0.1947208765169149</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02642434937081405</v>
+        <v>0.1142900616208657</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1899461241907346</v>
+        <v>-0.07996550731728209</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.3253798110098939</v>
+        <v>-0.09030309091146016</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6209229882480882</v>
+        <v>0.6770001102411148</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.5386027681463373</v>
+        <v>-0.5267211585816504</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.002739919114523326</v>
+        <v>0.07398354078567898</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.2808466423828462</v>
+        <v>0.3869310895808433</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1730645369575851</v>
+        <v>0.197662054262022</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1185275942017392</v>
+        <v>0.01069025224594381</v>
       </c>
       <c r="L10" t="n">
-        <v>0.04818420984629731</v>
+        <v>0.03167803534774859</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.08495738097378254</v>
+        <v>-0.04052178950133555</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.03696007426439404</v>
+        <v>-0.01551979342083148</v>
       </c>
       <c r="O10" t="n">
-        <v>0.02688253688717646</v>
+        <v>-0.002638298977165218</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.05030568765392397</v>
+        <v>-0.02647787564886622</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.002503558755023043</v>
+        <v>0.02182811915855095</v>
       </c>
       <c r="R10" t="n">
-        <v>4.714427404414166e-17</v>
+        <v>-0.01558931066967581</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.741932572210066e-18</v>
+        <v>-0.004515803541760142</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3.326710733158675e-17</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1.994837726319832e-16</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-3.631162110438793e-19</v>
       </c>
     </row>
     <row r="11">
@@ -1391,58 +1535,67 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01704800663221426</v>
+        <v>0.01945234050520501</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.01387046717142662</v>
+        <v>0.2487745657712129</v>
       </c>
       <c r="D11" t="n">
-        <v>0.4504890553993778</v>
+        <v>-0.1172766748508</v>
       </c>
       <c r="E11" t="n">
-        <v>0.822713741140544</v>
+        <v>0.9021554026766411</v>
       </c>
       <c r="F11" t="n">
-        <v>0.209818547408313</v>
+        <v>-0.05476401436332062</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.09683489936000467</v>
+        <v>-0.1821026800913821</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.2320534188698802</v>
+        <v>-0.2465371506357021</v>
       </c>
       <c r="I11" t="n">
-        <v>0.05410169139493414</v>
+        <v>-0.02932578331740247</v>
       </c>
       <c r="J11" t="n">
-        <v>0.03058124496601571</v>
+        <v>0.07251201444174223</v>
       </c>
       <c r="K11" t="n">
-        <v>0.07565546440445299</v>
+        <v>-0.03820426250337181</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.00433322739309798</v>
+        <v>-0.03166417762050844</v>
       </c>
       <c r="M11" t="n">
-        <v>0.04837677753442463</v>
+        <v>0.06269232589488337</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.00474066212776272</v>
+        <v>-0.003853463395514163</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.0171023253864479</v>
+        <v>-0.01370513978859162</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.01270101257478836</v>
+        <v>-0.0168969508040959</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.006910389930513018</v>
+        <v>-0.006669448993357718</v>
       </c>
       <c r="R11" t="n">
-        <v>-8.131843795844208e-18</v>
+        <v>0.01050367482011047</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.966531034519136e-19</v>
+        <v>0.0002824091672427708</v>
+      </c>
+      <c r="T11" t="n">
+        <v>5.603275979348539e-17</v>
+      </c>
+      <c r="U11" t="n">
+        <v>3.232990329670574e-17</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-1.708073815638757e-19</v>
       </c>
     </row>
     <row r="12">
@@ -1452,58 +1605,67 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1459841024642718</v>
+        <v>0.1391960127288416</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4629768702051163</v>
+        <v>0.4689717740035152</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3741542627706067</v>
+        <v>0.3359439395562244</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.2444295012656766</v>
+        <v>-0.1619880434717695</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2978201095163178</v>
+        <v>-0.07259674066831864</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.2601646688682381</v>
+        <v>-0.04159540195538597</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1780144081675542</v>
+        <v>-0.1478146374085346</v>
       </c>
       <c r="I12" t="n">
-        <v>0.5649614841048378</v>
+        <v>-0.1172825635802157</v>
       </c>
       <c r="J12" t="n">
-        <v>0.08447459508722199</v>
+        <v>0.09275263426173125</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0591986944331687</v>
+        <v>-0.06514145548197439</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1239439324323447</v>
+        <v>-0.005737884399958476</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.1277578412065113</v>
+        <v>0.06650107093004387</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.003626734359654995</v>
+        <v>0.01549159365023589</v>
       </c>
       <c r="O12" t="n">
-        <v>-0.117601022123942</v>
+        <v>-0.06936783535586877</v>
       </c>
       <c r="P12" t="n">
-        <v>0.03368504729142317</v>
+        <v>-0.01412911363784535</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.00695287102821277</v>
+        <v>0.004726229902557061</v>
       </c>
       <c r="R12" t="n">
-        <v>3.913531433406315e-17</v>
+        <v>0.006310102660923737</v>
       </c>
       <c r="S12" t="n">
-        <v>2.780358255201802e-18</v>
+        <v>-0.001192903961291455</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.7426922909895974</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-0.06911587770083695</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-0.0009706436424008907</v>
       </c>
     </row>
     <row r="13">
@@ -1513,424 +1675,697 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1104316274010218</v>
+        <v>0.1033628812193523</v>
       </c>
       <c r="C13" t="n">
-        <v>0.6860366211456691</v>
+        <v>0.1681321672842113</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03349114111918803</v>
+        <v>0.6501785114835269</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.04231802142345038</v>
+        <v>0.04322378083140358</v>
       </c>
       <c r="F13" t="n">
-        <v>0.05453306656975156</v>
+        <v>0.1394137451512065</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3499340246405621</v>
+        <v>0.3538771102427458</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.1666666869021749</v>
+        <v>-0.1671810515121961</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.4434284523013569</v>
+        <v>0.2947112743098896</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.01528236356806106</v>
+        <v>0.1082916597111276</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2816679927101474</v>
+        <v>-0.1428706886239224</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.08661219746532382</v>
+        <v>-0.1211049057969129</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2727373363763821</v>
+        <v>0.2273798880398999</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.03691371423464603</v>
+        <v>-0.01667624232015093</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.01580886981242715</v>
+        <v>-0.06587584152074234</v>
       </c>
       <c r="P13" t="n">
-        <v>-0.0007407421498174043</v>
+        <v>-0.009852762201890315</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.03662044978759676</v>
+        <v>-0.002467480526773911</v>
       </c>
       <c r="R13" t="n">
-        <v>1.066883942035045e-16</v>
+        <v>0.03523582528102373</v>
       </c>
       <c r="S13" t="n">
-        <v>-9.789657253989965e-19</v>
+        <v>0.004090309112690564</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-0.413533838795523</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.03848397859262177</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.0005404580018053893</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>saturated_ring_count</t>
+          <t>aliphatic_ring_count</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1574095132803282</v>
+        <v>0.1169515339885039</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.2789863420209398</v>
+        <v>0.5376856226652144</v>
       </c>
       <c r="D14" t="n">
-        <v>0.4614046606155013</v>
+        <v>-0.03735582632764256</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.06770088913245997</v>
+        <v>-0.2665188093652852</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.5312051927363706</v>
+        <v>-0.2151899523660121</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1703373673386153</v>
+        <v>-0.3418385866206299</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3183741187018993</v>
+        <v>-0.07839574184820752</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.3471101729189591</v>
+        <v>-0.4030673005936491</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.02308352528657881</v>
+        <v>0.04649148946620426</v>
       </c>
       <c r="K14" t="n">
-        <v>0.2190299056085784</v>
+        <v>0.02064116745775853</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.0245748827045706</v>
+        <v>0.08837458994371591</v>
       </c>
       <c r="M14" t="n">
-        <v>0.298315334262033</v>
+        <v>-0.08609856454939953</v>
       </c>
       <c r="N14" t="n">
-        <v>0.06117146416031094</v>
+        <v>0.03549233251251218</v>
       </c>
       <c r="O14" t="n">
-        <v>0.03559201754943536</v>
+        <v>-0.04682452039960408</v>
       </c>
       <c r="P14" t="n">
-        <v>0.05788049477251483</v>
+        <v>-0.01238093688803723</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.02020059752532793</v>
+        <v>0.008738266584171671</v>
       </c>
       <c r="R14" t="n">
-        <v>2.471024559029048e-17</v>
+        <v>-0.01906524708317944</v>
       </c>
       <c r="S14" t="n">
-        <v>2.520239071327296e-18</v>
+        <v>-0.004971254423638934</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-0.5184690996576102</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.04824938580667269</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.0006776005910784632</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>fraction_csp3</t>
+          <t>saturated_ring_count</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.130560220826499</v>
+        <v>0.1494329315982883</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.3842805117841873</v>
+        <v>0.3593972113211033</v>
       </c>
       <c r="D15" t="n">
-        <v>0.4419636458202623</v>
+        <v>-0.3885716247391399</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.3335385439400238</v>
+        <v>-0.06208696886615269</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2122697119232503</v>
+        <v>-0.3573302668009706</v>
       </c>
       <c r="G15" t="n">
-        <v>0.6048769216126003</v>
+        <v>0.1142667104929374</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.3084525937633167</v>
+        <v>0.3693079184839553</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1434479931920605</v>
+        <v>0.5091002204306506</v>
       </c>
       <c r="J15" t="n">
-        <v>0.02604490905255877</v>
+        <v>-0.03239374228443239</v>
       </c>
       <c r="K15" t="n">
-        <v>0.01271663244765648</v>
+        <v>-0.08529840815406617</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.0209227836191545</v>
+        <v>-0.1143973476691472</v>
       </c>
       <c r="M15" t="n">
-        <v>0.01743729010933593</v>
+        <v>0.3535974171226477</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0158810577565866</v>
+        <v>0.05165481945394394</v>
       </c>
       <c r="O15" t="n">
-        <v>0.01236076998097736</v>
+        <v>0.03509995091695709</v>
       </c>
       <c r="P15" t="n">
-        <v>0.0009329300448181222</v>
+        <v>0.07111727806758442</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.007752628782013518</v>
+        <v>-0.01608017607606163</v>
       </c>
       <c r="R15" t="n">
-        <v>-1.223742408148006e-17</v>
+        <v>0.03947704172634969</v>
       </c>
       <c r="S15" t="n">
-        <v>2.929999722519866e-19</v>
+        <v>0.0113845430891357</v>
+      </c>
+      <c r="T15" t="n">
+        <v>-2.197981031682564e-16</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-7.878042594923553e-16</v>
+      </c>
+      <c r="V15" t="n">
+        <v>4.105051581703353e-18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>heteroatom_count</t>
+          <t>fraction_csp3</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.2915584688705216</v>
+        <v>0.120442593006034</v>
       </c>
       <c r="C16" t="n">
-        <v>0.002972639682442009</v>
+        <v>0.2293937150253569</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.05664805820759385</v>
+        <v>-0.5019087410377764</v>
       </c>
       <c r="E16" t="n">
-        <v>0.05850826404176694</v>
+        <v>-0.1001027667902314</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0508321875636851</v>
+        <v>0.4219392869552414</v>
       </c>
       <c r="G16" t="n">
-        <v>0.03775455538641893</v>
+        <v>0.5717647031230226</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.04985801051077755</v>
+        <v>-0.3452646227810625</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.1442747398201829</v>
+        <v>-0.1902121542343134</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.05102601931783927</v>
+        <v>0.09214891560797711</v>
       </c>
       <c r="K16" t="n">
-        <v>0.001407626665510237</v>
+        <v>-0.01848456342181916</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.1342262798213341</v>
+        <v>-0.02104275385753028</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.3367260262806848</v>
+        <v>0.01197928397287122</v>
       </c>
       <c r="N16" t="n">
-        <v>0.7376709754439493</v>
+        <v>0.007813154427482996</v>
       </c>
       <c r="O16" t="n">
-        <v>-0.3233140063470171</v>
+        <v>0.02229974588034855</v>
       </c>
       <c r="P16" t="n">
-        <v>-0.02380177920346433</v>
+        <v>0.01079368006267247</v>
       </c>
       <c r="Q16" t="n">
-        <v>-0.312695662330911</v>
+        <v>-0.01508913359244017</v>
       </c>
       <c r="R16" t="n">
-        <v>-2.364482981367199e-16</v>
+        <v>0.01676042937497351</v>
       </c>
       <c r="S16" t="n">
-        <v>2.600679416457928e-17</v>
+        <v>0.000609984615829744</v>
+      </c>
+      <c r="T16" t="n">
+        <v>-3.692844564889605e-17</v>
+      </c>
+      <c r="U16" t="n">
+        <v>-1.084069289465105e-16</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1.651027499764809e-18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>formal_charge</t>
+          <t>heteroatom_count</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0</v>
+        <v>0.2672545038307104</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>-0.06801401440798331</v>
       </c>
       <c r="D17" t="n">
-        <v>-0</v>
+        <v>0.01803844196155891</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>0.02212073368700106</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>-0.06562201754760619</v>
       </c>
       <c r="G17" t="n">
-        <v>-0</v>
+        <v>0.03794531632115726</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>-0.08421072891765949</v>
       </c>
       <c r="I17" t="n">
-        <v>-0</v>
+        <v>0.1098365672813485</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>-0.07755912412221816</v>
       </c>
       <c r="K17" t="n">
-        <v>-0</v>
+        <v>0.0154062470375201</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>-0.03974480717829344</v>
       </c>
       <c r="M17" t="n">
-        <v>-0</v>
+        <v>-0.2339542921445813</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>0.8163866983574077</v>
       </c>
       <c r="O17" t="n">
-        <v>-0</v>
+        <v>0.009156403823679255</v>
       </c>
       <c r="P17" t="n">
-        <v>-0</v>
+        <v>-0.2520956501089904</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>-0.1678932337616305</v>
       </c>
       <c r="R17" t="n">
-        <v>1.869083786296133e-05</v>
+        <v>-0.2711017576197549</v>
       </c>
       <c r="S17" t="n">
-        <v>0.9999999998253263</v>
+        <v>0.06211415115907161</v>
+      </c>
+      <c r="T17" t="n">
+        <v>-1.479201232252398e-15</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-1.414532447929762e-15</v>
+      </c>
+      <c r="V17" t="n">
+        <v>4.637670339827865e-17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>atom_count</t>
+          <t>formal_charge</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.2925300997828106</v>
+        <v>-0</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01230617664597989</v>
+        <v>-0</v>
       </c>
       <c r="D18" t="n">
-        <v>0.003162235340474948</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0.04364090383615488</v>
+        <v>-0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.01760419526273392</v>
+        <v>-1.504632769052528e-36</v>
       </c>
       <c r="G18" t="n">
-        <v>0.04639472778792766</v>
+        <v>-0</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1721191329674828</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0.05992799386784295</v>
+        <v>-5.169878828456423e-26</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.05706901328501703</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.09095786880484345</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.2773625019867738</v>
+        <v>-0</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.01500630001870575</v>
+        <v>-0</v>
       </c>
       <c r="N18" t="n">
-        <v>-0.3714118780495696</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>-0.1531105925557026</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>-0.1143650729856704</v>
+        <v>-0</v>
       </c>
       <c r="Q18" t="n">
-        <v>-0.336937787026065</v>
+        <v>-3.469446951953614e-17</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.7071067810630348</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>1.321641819893289e-05</v>
+        <v>2.220446049250313e-16</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.002234312764177454</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.00996607253896549</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.9999478412620431</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>atom_count</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2689018855020133</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.02109358149891207</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.01253076280834863</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.04587546970958119</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.008603992765355698</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.03251380724996245</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.1249087118507631</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0.06506594776549258</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-0.07584945771070471</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.02771380294190151</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-0.194857615342596</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-0.1125578627028415</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-0.2665807363489315</v>
+      </c>
+      <c r="O19" t="n">
+        <v>-0.1704446136440045</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.0402350192833928</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>-0.4168969100844223</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-0.2487724230658879</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-0.0971189776514402</v>
+      </c>
+      <c r="T19" t="n">
+        <v>-0.06550849419106043</v>
+      </c>
+      <c r="U19" t="n">
+        <v>-0.7040293505986623</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.007163147663102124</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>amide_bond_count</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0.2794930408770562</v>
-      </c>
-      <c r="C19" t="n">
-        <v>-0.05178835273945064</v>
-      </c>
-      <c r="D19" t="n">
-        <v>-0.1386128557567501</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.1433774606307089</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.1659779675112449</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.199820489513011</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.06174272769044182</v>
-      </c>
-      <c r="I19" t="n">
-        <v>-0.1211035030387539</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.6930940089354309</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.1317662074658238</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0.4011947542246556</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-0.3165978835136729</v>
-      </c>
-      <c r="N19" t="n">
-        <v>-0.1799077736315904</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0.04574590700776476</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0.006099585737357627</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>-0.006786806505451783</v>
-      </c>
-      <c r="R19" t="n">
-        <v>5.431918717100666e-16</v>
-      </c>
-      <c r="S19" t="n">
-        <v>-5.634533827638617e-18</v>
+      <c r="B20" t="n">
+        <v>0.2553797388294077</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-0.1356345286102823</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.003512148507716183</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.04850830126530269</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-0.2214274974530389</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.1520162033327346</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.0829500382361775</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.06314101381672305</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.7451538779961672</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.2459772950055952</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.4142069511025882</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-0.145068399400119</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-0.05336658966988521</v>
+      </c>
+      <c r="O20" t="n">
+        <v>-0.1123271994365523</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.07257455661524082</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.03154399325392646</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-0.02570347384168966</v>
+      </c>
+      <c r="S20" t="n">
+        <v>-0.01590574181877194</v>
+      </c>
+      <c r="T20" t="n">
+        <v>-9.258890668063334e-17</v>
+      </c>
+      <c r="U20" t="n">
+        <v>1.151962639055337e-16</v>
+      </c>
+      <c r="V20" t="n">
+        <v>-8.160477507876661e-18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>molar_refractivity</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.2683494886484023</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.01999177747270206</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.005675697227679483</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.0627473026731126</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.005163760176944037</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.07545655059459533</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.165681874732303</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-0.09437440104493118</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-0.0635155319028078</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-0.02515164169547157</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-0.159095562809774</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-0.02713348690472258</v>
+      </c>
+      <c r="N21" t="n">
+        <v>-0.1542531715530171</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.005632694110671712</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.2955980965659628</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.7151998851388566</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-0.4244137559028076</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-0.2190564076824024</v>
+      </c>
+      <c r="T21" t="n">
+        <v>3.880219534581092e-15</v>
+      </c>
+      <c r="U21" t="n">
+        <v>6.765830273489758e-15</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-3.354249877828675e-17</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>labute_surface_area</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.2688506166482</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-0.01717377568265096</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.008519332102166112</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.05116679681928764</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.001764540041930193</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.0470590131700202</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.136371393221756</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-0.05563774055059783</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-0.08095145710061126</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.01346657257803495</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-0.1128801129192198</v>
+      </c>
+      <c r="M22" t="n">
+        <v>-0.171914311571688</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-0.1428618049804945</v>
+      </c>
+      <c r="O22" t="n">
+        <v>-0.1295525787667646</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-0.2030632969533575</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.1153811744355907</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.2764034239099855</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.8268329539488324</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-1.686418268269791e-14</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-1.882839019843949e-14</v>
+      </c>
+      <c r="V22" t="n">
+        <v>1.029800136040481e-17</v>
       </c>
     </row>
   </sheetData>
@@ -1944,7 +2379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2043,6 +2478,21 @@
           <t>PC18</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>PC19</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>PC20</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>PC21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2051,58 +2501,67 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8060893486564648</v>
+        <v>0.9185912924122391</v>
       </c>
       <c r="C2" t="n">
-        <v>3.109116747481643</v>
+        <v>1.307735493583924</v>
       </c>
       <c r="D2" t="n">
-        <v>1.280938698223757</v>
+        <v>2.743830813164687</v>
       </c>
       <c r="E2" t="n">
-        <v>1.363016174111248</v>
+        <v>2.120237063892279</v>
       </c>
       <c r="F2" t="n">
-        <v>0.589611366955669</v>
+        <v>0.5761158324192267</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7413091839353565</v>
+        <v>0.880255265999527</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.4066551696087257</v>
+        <v>-0.4338992823676587</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.3325234916517621</v>
+        <v>0.3662957568515329</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.04168547218930086</v>
+        <v>0.01658228745589798</v>
       </c>
       <c r="K2" t="n">
-        <v>0.009413196171431272</v>
+        <v>-0.04931189689078631</v>
       </c>
       <c r="L2" t="n">
-        <v>0.05444071131203111</v>
+        <v>0.07372414832961256</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.05295420387415754</v>
+        <v>-0.04566335924212025</v>
       </c>
       <c r="N2" t="n">
-        <v>0.02438832283379606</v>
+        <v>0.01484733273659468</v>
       </c>
       <c r="O2" t="n">
-        <v>0.04628052117523295</v>
+        <v>0.04842914025421502</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.0161108089732519</v>
+        <v>0.001495910415408344</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.004074476258075131</v>
+        <v>0.01574696301467695</v>
       </c>
       <c r="R2" t="n">
-        <v>3.288361233392808e-18</v>
+        <v>-0.00164389156809364</v>
       </c>
       <c r="S2" t="n">
-        <v>2.429449265480645e-19</v>
+        <v>-4.334798931238209e-05</v>
+      </c>
+      <c r="T2" t="n">
+        <v>7.854264458333126e-17</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-6.581061097994106e-19</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1.098174346064245e-19</v>
       </c>
     </row>
     <row r="3">
@@ -2112,58 +2571,67 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.006371808474067</v>
+        <v>3.198620743453328</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.2171201598511673</v>
+        <v>-1.063271339527957</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.7481217262986636</v>
+        <v>0.03227254714175377</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.302885353827357</v>
+        <v>-0.2691250292349991</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1748757342037966</v>
+        <v>0.2745417156597193</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1840095657279615</v>
+        <v>0.2433763672443794</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.5139790821498222</v>
+        <v>-0.4599237514627103</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.2911392182700051</v>
+        <v>0.4007440201472231</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1244395839170855</v>
+        <v>0.1714427047185607</v>
       </c>
       <c r="K3" t="n">
-        <v>0.01172393934693383</v>
+        <v>0.04193668569974989</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.1270033120166539</v>
+        <v>-0.1142844383472808</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.06868326802888723</v>
+        <v>-0.1129774025593509</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.0968338443379058</v>
+        <v>-0.06799583001931189</v>
       </c>
       <c r="O3" t="n">
-        <v>0.000232375253969917</v>
+        <v>-0.05013831022681962</v>
       </c>
       <c r="P3" t="n">
-        <v>0.02561222057291286</v>
+        <v>0.04331393320946185</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.009873073019003418</v>
+        <v>-0.006886122200161717</v>
       </c>
       <c r="R3" t="n">
-        <v>-2.984349716976627e-17</v>
+        <v>-0.007820460380782119</v>
       </c>
       <c r="S3" t="n">
-        <v>-2.516781312125146e-20</v>
+        <v>0.0001138272026954735</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-2.290439765325714e-17</v>
+      </c>
+      <c r="U3" t="n">
+        <v>3.703062811542186e-17</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1.917658174422278e-19</v>
       </c>
     </row>
     <row r="4">
@@ -2173,58 +2641,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.256617973845516</v>
+        <v>-2.571219240255914</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.538472918442241</v>
+        <v>-1.322354543721455</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.8596482247773115</v>
+        <v>-1.219205502384599</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1438192032433255</v>
+        <v>-0.270665895194926</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1873183420424393</v>
+        <v>0.07246710535636333</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3760122196969505</v>
+        <v>0.2101823781311334</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.4435173314846487</v>
+        <v>-0.4435231724109035</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2237897541390827</v>
+        <v>-0.2716944906776979</v>
       </c>
       <c r="J4" t="n">
-        <v>0.09189049516590878</v>
+        <v>0.1224925394107584</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.08625118735339121</v>
+        <v>0.08060232850609189</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.1326646252164199</v>
+        <v>-0.1251763047870517</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01145106103936953</v>
+        <v>-0.05280215436014954</v>
       </c>
       <c r="N4" t="n">
-        <v>0.05066483196673446</v>
+        <v>0.006125625212424252</v>
       </c>
       <c r="O4" t="n">
-        <v>0.01051372623262077</v>
+        <v>0.0567086336491807</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.01662877151874494</v>
+        <v>-0.0306044211479324</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.003243314685652564</v>
+        <v>0.01187681834903105</v>
       </c>
       <c r="R4" t="n">
-        <v>2.531948349518272e-18</v>
+        <v>-0.00223439801232002</v>
       </c>
       <c r="S4" t="n">
-        <v>8.747132786346075e-19</v>
+        <v>0.001034233698855962</v>
+      </c>
+      <c r="T4" t="n">
+        <v>3.415852173030542e-17</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3.699367381244622e-18</v>
+      </c>
+      <c r="V4" t="n">
+        <v>4.789901869553547e-20</v>
       </c>
     </row>
     <row r="5">
@@ -2234,58 +2711,67 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.77283914641589</v>
+        <v>13.93074989501791</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.3655072045019341</v>
+        <v>-3.434195400477437</v>
       </c>
       <c r="D5" t="n">
-        <v>-2.405830699539361</v>
+        <v>0.3888953211116767</v>
       </c>
       <c r="E5" t="n">
-        <v>0.06481190252167589</v>
+        <v>0.2884611021883105</v>
       </c>
       <c r="F5" t="n">
-        <v>2.014236966984853</v>
+        <v>1.628423494905658</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2165048501057488</v>
+        <v>-0.6026232705225146</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2310984980022156</v>
+        <v>0.2545400386205397</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1521768857782673</v>
+        <v>-0.2164597653764913</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.04137447198101765</v>
+        <v>0.02715080351406178</v>
       </c>
       <c r="K5" t="n">
-        <v>0.03637871794974707</v>
+        <v>-0.07131555192146601</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0266913101852161</v>
+        <v>0.02154753704204188</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0151968072412153</v>
+        <v>0.02857294342166069</v>
       </c>
       <c r="N5" t="n">
-        <v>0.01956859643833346</v>
+        <v>0.01258771593211679</v>
       </c>
       <c r="O5" t="n">
-        <v>0.007775384306031734</v>
+        <v>0.01652307718064179</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.0006017871373042573</v>
+        <v>-0.0008209921339881113</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0006184965974638201</v>
+        <v>0.001946828746876778</v>
       </c>
       <c r="R5" t="n">
-        <v>-1.3172129212778e-17</v>
+        <v>1.04214086094544e-05</v>
       </c>
       <c r="S5" t="n">
-        <v>2.143049361653997e-20</v>
+        <v>-4.595688435788099e-05</v>
+      </c>
+      <c r="T5" t="n">
+        <v>3.250262778430699e-17</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-3.736713957133228e-19</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3.115012391042553e-19</v>
       </c>
     </row>
     <row r="6">
@@ -2295,58 +2781,67 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.1377555482349118</v>
+        <v>0.1094112080819708</v>
       </c>
       <c r="C6" t="n">
-        <v>-1.485878083901734</v>
+        <v>2.884639816939076</v>
       </c>
       <c r="D6" t="n">
-        <v>3.81372352227048</v>
+        <v>-2.433744220173227</v>
       </c>
       <c r="E6" t="n">
-        <v>2.413245890988593</v>
+        <v>3.314887788529611</v>
       </c>
       <c r="F6" t="n">
-        <v>1.191065058134873</v>
+        <v>0.5471720761737034</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.4970510074769629</v>
+        <v>-0.7314008750593113</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1384598443174148</v>
+        <v>0.1283516137417079</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1408748173898609</v>
+        <v>-0.1691862235265929</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1362892353152107</v>
+        <v>0.05740617144123597</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.0572939354162253</v>
+        <v>0.1330793146057737</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.04319132543526153</v>
+        <v>-0.03695522780260656</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.02304631017714869</v>
+        <v>-0.03680780643384632</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.01185311745226131</v>
+        <v>-0.004882832654869794</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.004298381272866554</v>
+        <v>-0.01064633332741424</v>
       </c>
       <c r="P6" t="n">
-        <v>0.006188184079570742</v>
+        <v>0.007059645364873248</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.002659444604536469</v>
+        <v>-0.002365129056801819</v>
       </c>
       <c r="R6" t="n">
-        <v>-1.518131082280446e-17</v>
+        <v>-0.00196685763422226</v>
       </c>
       <c r="S6" t="n">
-        <v>1.161544165704909e-19</v>
+        <v>0.000178408028554587</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2.041851103814967e-17</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-1.199130553995843e-17</v>
+      </c>
+      <c r="V6" t="n">
+        <v>7.145582196026837e-19</v>
       </c>
     </row>
     <row r="7">
@@ -2356,58 +2851,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.520551066117406</v>
+        <v>-2.850596719821731</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.782521544794057</v>
+        <v>-1.743425184144358</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.690026416550172</v>
+        <v>-0.229259530516429</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5110938337593499</v>
+        <v>-0.07275579449015264</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2582207626623423</v>
+        <v>-0.7842093797319257</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.7997779715525806</v>
+        <v>-0.9063682071628786</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1242074306034454</v>
+        <v>0.1954994473638497</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.1489665433363107</v>
+        <v>0.2025965372355335</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.1425208570586057</v>
+        <v>-0.1359651608859568</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.08714045425602941</v>
+        <v>-0.05124235976833878</v>
       </c>
       <c r="L7" t="n">
-        <v>0.03924530311401394</v>
+        <v>0.1075479563065601</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.2084168580701999</v>
+        <v>-0.2223753460463933</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.002222200885448973</v>
+        <v>0.02567849290909656</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.007411270505783404</v>
+        <v>-0.0197753486497849</v>
       </c>
       <c r="P7" t="n">
-        <v>0.001749930623049917</v>
+        <v>-0.001682414883488275</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.01522092085211142</v>
+        <v>0.01122883031139844</v>
       </c>
       <c r="R7" t="n">
-        <v>-1.300025473750682e-17</v>
+        <v>0.01335146785891038</v>
       </c>
       <c r="S7" t="n">
-        <v>2.182277704842821e-19</v>
+        <v>0.001021985533227659</v>
+      </c>
+      <c r="T7" t="n">
+        <v>5.984380596823297e-17</v>
+      </c>
+      <c r="U7" t="n">
+        <v>8.896296240138542e-18</v>
+      </c>
+      <c r="V7" t="n">
+        <v>2.290908934362495e-19</v>
       </c>
     </row>
     <row r="8">
@@ -2417,58 +2921,67 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.1110681882476334</v>
+        <v>-0.05061845354061949</v>
       </c>
       <c r="C8" t="n">
-        <v>-2.119347807969487</v>
+        <v>1.364751209088487</v>
       </c>
       <c r="D8" t="n">
-        <v>1.850866062572223</v>
+        <v>-2.592451144189534</v>
       </c>
       <c r="E8" t="n">
-        <v>-1.555210541032255</v>
+        <v>-0.8834451696064116</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5678997101193722</v>
+        <v>1.268141181325095</v>
       </c>
       <c r="G8" t="n">
-        <v>0.08255300464111467</v>
+        <v>0.2824081201312288</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3274088696345455</v>
+        <v>0.412734438426021</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.2982305373676555</v>
+        <v>0.3568074955229987</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.1063034626322029</v>
+        <v>-0.1132265793690523</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.05730418572840406</v>
+        <v>-0.02052408715541879</v>
       </c>
       <c r="L8" t="n">
-        <v>0.07493495103590057</v>
+        <v>0.1027991853080473</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.0004581766595494357</v>
+        <v>-0.003146318178162862</v>
       </c>
       <c r="N8" t="n">
-        <v>0.02432707836140304</v>
+        <v>0.002999803298563717</v>
       </c>
       <c r="O8" t="n">
-        <v>0.03207062952949603</v>
+        <v>0.05145568170725172</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.02042433010294729</v>
+        <v>-0.0002009285799631744</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.01265667150165609</v>
+        <v>-0.02008075710427028</v>
       </c>
       <c r="R8" t="n">
-        <v>-3.950071085101069e-17</v>
+        <v>-0.004961171917919767</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.273249148359293e-19</v>
+        <v>0.001571932182116409</v>
+      </c>
+      <c r="T8" t="n">
+        <v>5.22242388491097e-17</v>
+      </c>
+      <c r="U8" t="n">
+        <v>3.969122182052326e-17</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-2.239487126800382e-19</v>
       </c>
     </row>
     <row r="9">
@@ -2478,58 +2991,67 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.7197201034718054</v>
+        <v>-0.7498571665275597</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.0157058766724529</v>
+        <v>0.5740764137995966</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1577826941065335</v>
+        <v>-0.0737687100038055</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.6178350029706348</v>
+        <v>-0.7043540388845267</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1732983753821617</v>
+        <v>-0.01876603580181559</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.105066332917976</v>
+        <v>-0.1398842055898149</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.2774923765000177</v>
+        <v>-0.2890910515801601</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1383212268153416</v>
+        <v>-0.1085685380514362</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.18957610736386</v>
+        <v>-0.1190544070525426</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.01797374434444253</v>
+        <v>-0.1249666233055339</v>
       </c>
       <c r="L9" t="n">
-        <v>0.02681660987362441</v>
+        <v>0.0247474881606</v>
       </c>
       <c r="M9" t="n">
-        <v>0.07240467751889153</v>
+        <v>0.05337960605355868</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.03252975859314797</v>
+        <v>-0.05890131078602342</v>
       </c>
       <c r="O9" t="n">
-        <v>0.01624165483340757</v>
+        <v>0.01489786710013665</v>
       </c>
       <c r="P9" t="n">
-        <v>0.01033509912083287</v>
+        <v>0.02096520089082227</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.005876269024626171</v>
+        <v>-0.008996608802363602</v>
       </c>
       <c r="R9" t="n">
-        <v>3.137429028865497e-17</v>
+        <v>0.0117576758570474</v>
       </c>
       <c r="S9" t="n">
-        <v>1.579289617549187e-18</v>
+        <v>9.70248938297918e-05</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-3.30701839652837e-17</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-4.849448488244168e-18</v>
+      </c>
+      <c r="V9" t="n">
+        <v>5.563032197412103e-19</v>
       </c>
     </row>
     <row r="10">
@@ -2539,58 +3061,67 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.497044702126997</v>
+        <v>-1.708795050169325</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.1732047840846914</v>
+        <v>-0.9572491639398591</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.7439381983135327</v>
+        <v>0.08477779253507936</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1183356467910958</v>
+        <v>-0.09961424881082005</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1827400499279593</v>
+        <v>0.1869225455269203</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3684242877008134</v>
+        <v>0.3455699205649153</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1485283119861725</v>
+        <v>-0.1136269435907022</v>
       </c>
       <c r="I10" t="n">
-        <v>0.001724841371221122</v>
+        <v>-0.008206443286400685</v>
       </c>
       <c r="J10" t="n">
-        <v>0.01989830242778603</v>
+        <v>0.123239162414297</v>
       </c>
       <c r="K10" t="n">
-        <v>0.09288209036009182</v>
+        <v>-0.08237977496191418</v>
       </c>
       <c r="L10" t="n">
-        <v>0.005846652868646919</v>
+        <v>-0.02474075051758863</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0354575662888072</v>
+        <v>0.03902458458166776</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.04942313076411104</v>
+        <v>-0.05515174611958255</v>
       </c>
       <c r="O10" t="n">
-        <v>-0.03984858039754566</v>
+        <v>-0.03843506188400815</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.04606652613246146</v>
+        <v>-0.0586269132109169</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.001472202868048293</v>
+        <v>-0.004418268052475549</v>
       </c>
       <c r="R10" t="n">
-        <v>2.549981549646863e-17</v>
+        <v>-0.001515579080804934</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.410793356986903e-18</v>
+        <v>0.002858742908259826</v>
+      </c>
+      <c r="T10" t="n">
+        <v>7.683075053266087e-17</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-8.511759453889208e-18</v>
+      </c>
+      <c r="V10" t="n">
+        <v>7.813226344129639e-19</v>
       </c>
     </row>
     <row r="11">
@@ -2600,58 +3131,67 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-1.969130657614917</v>
+        <v>-2.171327735838608</v>
       </c>
       <c r="C11" t="n">
-        <v>0.943539925247452</v>
+        <v>-0.6440260259569325</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.7596206367931251</v>
+        <v>1.18805601089914</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1337117508352408</v>
+        <v>0.1082646540430787</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.07403020857614677</v>
+        <v>-0.1021137452503711</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1153815181970236</v>
+        <v>0.21937492903041</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4293041542414215</v>
+        <v>0.4839843213610238</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.1401563555171501</v>
+        <v>0.1464826890062219</v>
       </c>
       <c r="J11" t="n">
-        <v>0.008429939735171232</v>
+        <v>-0.02075150571799979</v>
       </c>
       <c r="K11" t="n">
-        <v>0.06156697036107306</v>
+        <v>-0.002029671644268191</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.2076567611287644</v>
+        <v>-0.209566853409544</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.00720015067614148</v>
+        <v>-0.02823144866820041</v>
       </c>
       <c r="N11" t="n">
-        <v>0.07031489109538705</v>
+        <v>0.09078674742469305</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.01464475322703016</v>
+        <v>0.01026944265741648</v>
       </c>
       <c r="P11" t="n">
-        <v>0.01230576607415479</v>
+        <v>0.008772301651953748</v>
       </c>
       <c r="Q11" t="n">
-        <v>-0.005229162616819596</v>
+        <v>-0.02688137141663093</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.218249057114873e-17</v>
+        <v>0.006131730505336411</v>
       </c>
       <c r="S11" t="n">
-        <v>-6.956076262717698e-19</v>
+        <v>-0.000489664690745313</v>
+      </c>
+      <c r="T11" t="n">
+        <v>7.979404272028422e-17</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-9.628105520583778e-18</v>
+      </c>
+      <c r="V11" t="n">
+        <v>5.978055390679006e-19</v>
       </c>
     </row>
     <row r="12">
@@ -2661,115 +3201,133 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.3128864053420523</v>
+        <v>-0.03320676553119016</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9227405557195976</v>
+        <v>2.690660939962605</v>
       </c>
       <c r="D12" t="n">
-        <v>1.556651528663652</v>
+        <v>0.4029454784398798</v>
       </c>
       <c r="E12" t="n">
-        <v>-1.128543476568866</v>
+        <v>-1.036234368408641</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.4327450082313611</v>
+        <v>0.03302185595819862</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04346658778523278</v>
+        <v>0.0441643102584004</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4268265345368618</v>
+        <v>0.4167542300815099</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4496948743444826</v>
+        <v>-0.5611374664683201</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.07253297166681713</v>
+        <v>0.05220667334756991</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1902954231980766</v>
+        <v>-0.2112733915352922</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.07286333633669674</v>
+        <v>-0.09359922854615188</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.09162267112490832</v>
+        <v>-0.05849518442543333</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.04240768912729317</v>
+        <v>-0.005182729916700558</v>
       </c>
       <c r="O12" t="n">
-        <v>0.04309593376409152</v>
+        <v>-0.005628815378450186</v>
       </c>
       <c r="P12" t="n">
-        <v>0.002006029613941106</v>
+        <v>0.03560486303552809</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.0001212533674676183</v>
+        <v>0.01684117592885986</v>
       </c>
       <c r="R12" t="n">
-        <v>-1.137625440373282e-17</v>
+        <v>-0.005869548143013977</v>
       </c>
       <c r="S12" t="n">
-        <v>-3.987373176412628e-19</v>
+        <v>0.0009426441391058254</v>
+      </c>
+      <c r="T12" t="n">
+        <v>4.746935231784422e-17</v>
+      </c>
+      <c r="U12" t="n">
+        <v>1.591971635151751e-17</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-2.099502055299488e-19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>-1.317579605158018</v>
+        <v>-1.390101661639554</v>
       </c>
       <c r="C13" t="n">
-        <v>1.018372997503429</v>
+        <v>0.107180964311897</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.4306020589299386</v>
+        <v>1.12164459452389</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.133572613858968</v>
+        <v>-0.2899372108417368</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.225734416804669</v>
+        <v>-0.224454357346138</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1883921174227255</v>
+        <v>0.1267602441738264</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.01389278880086208</v>
+        <v>-0.05766152208343709</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2324135206389323</v>
+        <v>-0.3185757009624822</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.1769549848720554</v>
+        <v>-0.2047298717419787</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.1729075393725435</v>
+        <v>0.002811582529100678</v>
       </c>
       <c r="L13" t="n">
-        <v>0.02033892518580979</v>
+        <v>0.05618022462602379</v>
       </c>
       <c r="M13" t="n">
-        <v>0.02299916297882027</v>
+        <v>-0.02897793820425739</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.01864284426739579</v>
+        <v>-0.04756730896070348</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.01780875299812209</v>
+        <v>0.0007322326277221281</v>
       </c>
       <c r="P13" t="n">
-        <v>0.0123805231538932</v>
+        <v>0.002013536335394462</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.009774614881993786</v>
+        <v>-0.018629791265312</v>
       </c>
       <c r="R13" t="n">
-        <v>-5.211120618197549e-17</v>
+        <v>-0.003559790075564712</v>
       </c>
       <c r="S13" t="n">
-        <v>2.490307525445208e-18</v>
+        <v>4.930755173725667e-05</v>
+      </c>
+      <c r="T13" t="n">
+        <v>3.727874750831981e-18</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-3.572452407840199e-17</v>
+      </c>
+      <c r="V13" t="n">
+        <v>-3.437230514345623e-20</v>
       </c>
     </row>
     <row r="14">
@@ -2779,115 +3337,137 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-2.062348374473352</v>
+        <v>-0.7945806581652994</v>
       </c>
       <c r="C14" t="n">
-        <v>1.066563327733697</v>
+        <v>-1.330540083611993</v>
       </c>
       <c r="D14" t="n">
-        <v>-1.024143666791429</v>
+        <v>-0.7107805229801361</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2609243208506203</v>
+        <v>-0.1708058961391201</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2319575803460575</v>
+        <v>0.4583443871523153</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2456325632163362</v>
+        <v>0.2610664482545422</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3389663788635657</v>
+        <v>-0.4992208713878967</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.2460908632812842</v>
+        <v>-0.1711107603195468</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.01463529608779982</v>
+        <v>-0.4768004699850129</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.002566779960753053</v>
+        <v>0.2084366033598554</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.03074421410786141</v>
+        <v>-0.03102440084668579</v>
       </c>
       <c r="M14" t="n">
-        <v>0.1503666470835425</v>
+        <v>0.06737005923841211</v>
       </c>
       <c r="N14" t="n">
-        <v>-0.02353399811444229</v>
+        <v>0.06011068329962833</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0448335754209867</v>
+        <v>-0.04397105017711442</v>
       </c>
       <c r="P14" t="n">
-        <v>0.01954193686681036</v>
+        <v>0.01411877892035414</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.01095284342027528</v>
+        <v>0.009807463730898153</v>
       </c>
       <c r="R14" t="n">
-        <v>-4.1435362124519e-17</v>
+        <v>-0.003419596435871947</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.522737217618912e-18</v>
+        <v>0.0004893369771971028</v>
+      </c>
+      <c r="T14" t="n">
+        <v>8.173823339614346e-17</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1.78844011976625e-17</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.641937211342833e-20</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Glatiramer acetate</t>
+        </is>
+      </c>
       <c r="B15" t="n">
-        <v>-2.422319616999643</v>
+        <v>-2.302051971365755</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.2190987326891655</v>
+        <v>-0.7979091711611135</v>
       </c>
       <c r="D15" t="n">
-        <v>-1.536762529986881</v>
+        <v>1.3824578610102</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4125093178086977</v>
+        <v>0.07986378144101901</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.2789059679901754</v>
+        <v>-0.3612941404168278</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.6638310155721727</v>
+        <v>-0.1238947802905586</v>
       </c>
       <c r="H15" t="n">
-        <v>0.08335892048832241</v>
+        <v>0.4049683423840572</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.1420080619641978</v>
+        <v>0.3254763698087087</v>
       </c>
       <c r="J15" t="n">
-        <v>0.005059398902696044</v>
+        <v>-0.0904552592017193</v>
       </c>
       <c r="K15" t="n">
-        <v>0.04849915615776804</v>
+        <v>0.03885576412182973</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.06344696436343461</v>
+        <v>-0.06111911900280644</v>
       </c>
       <c r="M15" t="n">
-        <v>0.01016433669440362</v>
+        <v>0.1329662430586329</v>
       </c>
       <c r="N15" t="n">
-        <v>0.001635326562541076</v>
+        <v>-0.0558250400295003</v>
       </c>
       <c r="O15" t="n">
-        <v>0.01300783150569474</v>
+        <v>0.03383669511343422</v>
       </c>
       <c r="P15" t="n">
-        <v>-0.04368035719795745</v>
+        <v>0.03507319403682073</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.006680966502189327</v>
+        <v>0.0165936603988425</v>
       </c>
       <c r="R15" t="n">
-        <v>-5.012772950897007e-17</v>
+        <v>0.007414314484882764</v>
       </c>
       <c r="S15" t="n">
-        <v>2.402602164366244e-18</v>
+        <v>0.001147752702673417</v>
+      </c>
+      <c r="T15" t="n">
+        <v>-1.313107644430656e-18</v>
+      </c>
+      <c r="U15" t="n">
+        <v>3.244351475520919e-18</v>
+      </c>
+      <c r="V15" t="n">
+        <v>6.976076769947792e-19</v>
       </c>
     </row>
     <row r="16">
@@ -2897,58 +3477,67 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-1.225357113024292</v>
+        <v>-2.738033836841566</v>
       </c>
       <c r="C16" t="n">
-        <v>1.006842160552219</v>
+        <v>-1.484199085676446</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.3477149551900535</v>
+        <v>0.273896608776768</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.2755591390641861</v>
+        <v>-0.07424254149358921</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04521877247819586</v>
+        <v>-0.6861448141945697</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.04663886153584561</v>
+        <v>-0.7050053319914532</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.01508841182740166</v>
+        <v>0.1644599482016086</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1098600077343457</v>
+        <v>0.2413499033685579</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.1014345272179989</v>
+        <v>0.008583477624263251</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.1211854574480216</v>
+        <v>-0.02593841602701423</v>
       </c>
       <c r="L16" t="n">
-        <v>0.04136514836972682</v>
+        <v>-0.07871903884010013</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.01407382958812328</v>
+        <v>-0.0007532619796421337</v>
       </c>
       <c r="N16" t="n">
-        <v>-0.03477117288077908</v>
+        <v>-0.01326702144800457</v>
       </c>
       <c r="O16" t="n">
-        <v>-0.006077976004108659</v>
+        <v>0.0263216751175838</v>
       </c>
       <c r="P16" t="n">
-        <v>-0.00957145280266815</v>
+        <v>-0.03524046569902325</v>
       </c>
       <c r="Q16" t="n">
-        <v>-0.01086709694831974</v>
+        <v>0.002210195741729981</v>
       </c>
       <c r="R16" t="n">
-        <v>-4.027300729140997e-17</v>
+        <v>-0.01111708011463143</v>
       </c>
       <c r="S16" t="n">
-        <v>-4.054297156610868e-18</v>
+        <v>-0.001708477727932499</v>
+      </c>
+      <c r="T16" t="n">
+        <v>-2.742548410138669e-19</v>
+      </c>
+      <c r="U16" t="n">
+        <v>1.269526553351986e-17</v>
+      </c>
+      <c r="V16" t="n">
+        <v>-4.47609076043062e-19</v>
       </c>
     </row>
     <row r="17">
@@ -2958,58 +3547,67 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-1.936872763126338</v>
+        <v>-1.303681440824543</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3295468679414648</v>
+        <v>0.1579047107273379</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1057519562195742</v>
+        <v>1.086154631025582</v>
       </c>
       <c r="E17" t="n">
-        <v>2.020224441339073</v>
+        <v>-0.3300151582937069</v>
       </c>
       <c r="F17" t="n">
-        <v>0.5005080496119498</v>
+        <v>0.0760090550283523</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.1539972624210404</v>
+        <v>-0.1070069802080468</v>
       </c>
       <c r="H17" t="n">
-        <v>0.03898210869068159</v>
+        <v>-0.02482645043759143</v>
       </c>
       <c r="I17" t="n">
-        <v>0.08793137429068874</v>
+        <v>-0.1468495316892836</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.07115618035507396</v>
+        <v>-0.1170043094826653</v>
       </c>
       <c r="K17" t="n">
-        <v>0.02845903209685407</v>
+        <v>0.007556086437403329</v>
       </c>
       <c r="L17" t="n">
-        <v>0.007508692466188809</v>
+        <v>0.07023944035423729</v>
       </c>
       <c r="M17" t="n">
-        <v>0.1025453605113609</v>
+        <v>-0.04696215263039065</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.03047335432715342</v>
+        <v>-0.05445524002604605</v>
       </c>
       <c r="O17" t="n">
-        <v>-0.02460856361577184</v>
+        <v>-0.0004386864039762712</v>
       </c>
       <c r="P17" t="n">
-        <v>-0.003514772611255284</v>
+        <v>-0.009737765842462338</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.005156639203020045</v>
+        <v>-0.008942124943131558</v>
       </c>
       <c r="R17" t="n">
-        <v>-4.103936233986979e-17</v>
+        <v>-0.01047857400118125</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.684879061545644e-19</v>
+        <v>-0.001954877855687228</v>
+      </c>
+      <c r="T17" t="n">
+        <v>5.698979651271966e-17</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1.902077520630771e-17</v>
+      </c>
+      <c r="V17" t="n">
+        <v>1.113846527594784e-18</v>
       </c>
     </row>
     <row r="18">
@@ -3019,58 +3617,67 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.578184289753111</v>
+        <v>-2.115761437823045</v>
       </c>
       <c r="C18" t="n">
-        <v>2.073030557367749</v>
+        <v>-0.3510916094019023</v>
       </c>
       <c r="D18" t="n">
-        <v>1.234524428636279</v>
+        <v>0.3955972522422678</v>
       </c>
       <c r="E18" t="n">
-        <v>-1.258182289057655</v>
+        <v>2.147169051038296</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.4061928291566426</v>
+        <v>-0.2209347019967602</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.6795344076936661</v>
+        <v>-0.3300510012938923</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.3019107253623303</v>
+        <v>0.03265295623348146</v>
       </c>
       <c r="I18" t="n">
-        <v>0.02876876175262505</v>
+        <v>-0.1032821872814351</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1447194981741752</v>
+        <v>-0.05035439462972204</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.02346959933866152</v>
+        <v>-0.05759883444486207</v>
       </c>
       <c r="L18" t="n">
-        <v>0.00927521866568781</v>
+        <v>-0.01933123898117607</v>
       </c>
       <c r="M18" t="n">
-        <v>0.02658645860950509</v>
+        <v>0.0994533394008508</v>
       </c>
       <c r="N18" t="n">
-        <v>0.01043956838152001</v>
+        <v>-0.04457818371782512</v>
       </c>
       <c r="O18" t="n">
-        <v>-0.006231154752540411</v>
+        <v>-0.02154775183889097</v>
       </c>
       <c r="P18" t="n">
-        <v>-0.004556857599913921</v>
+        <v>-0.01303318379267847</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.001852498389093641</v>
+        <v>-0.008292699625667435</v>
       </c>
       <c r="R18" t="n">
-        <v>-2.971051184751426e-17</v>
+        <v>0.00887645428874503</v>
       </c>
       <c r="S18" t="n">
-        <v>4.27974603258717e-18</v>
+        <v>-0.0002794101271687591</v>
+      </c>
+      <c r="T18" t="n">
+        <v>6.816425861349608e-18</v>
+      </c>
+      <c r="U18" t="n">
+        <v>5.528824089774241e-17</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-6.77836332567464e-19</v>
       </c>
     </row>
     <row r="19">
@@ -3080,58 +3687,67 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-2.045528996678056</v>
+        <v>3.032466609852652</v>
       </c>
       <c r="C19" t="n">
-        <v>-1.702823965670773</v>
+        <v>2.765910706229713</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.7065201410182897</v>
+        <v>1.588945308003243</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.2786197923253201</v>
+        <v>-1.274939833886755</v>
       </c>
       <c r="F19" t="n">
-        <v>0.3391855124865656</v>
+        <v>0.06108116134064329</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5847275412116277</v>
+        <v>-0.6322677607806774</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.5401288664024988</v>
+        <v>-0.3130709522797612</v>
       </c>
       <c r="I19" t="n">
-        <v>0.2511258301870062</v>
+        <v>0.07852771202839144</v>
       </c>
       <c r="J19" t="n">
-        <v>0.07775043764950741</v>
+        <v>0.08025372323741393</v>
       </c>
       <c r="K19" t="n">
-        <v>-0.04398459496908277</v>
+        <v>0.1169627867654012</v>
       </c>
       <c r="L19" t="n">
-        <v>0.01536277103139732</v>
+        <v>-0.002573498038343154</v>
       </c>
       <c r="M19" t="n">
-        <v>-0.0154333848964265</v>
+        <v>0.03433604042412679</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0134565647623171</v>
+        <v>0.008001645520930398</v>
       </c>
       <c r="O19" t="n">
-        <v>0.02728834051835376</v>
+        <v>0.0001844442389023929</v>
       </c>
       <c r="P19" t="n">
-        <v>0.004599769238879711</v>
+        <v>-0.007242492758158435</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.01001143423801158</v>
+        <v>-0.004516909515085729</v>
       </c>
       <c r="R19" t="n">
-        <v>-6.706451582633748e-17</v>
+        <v>0.004039477869197611</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.271925805364323e-18</v>
+        <v>-0.0001828898036805001</v>
+      </c>
+      <c r="T19" t="n">
+        <v>2.494174955539895e-16</v>
+      </c>
+      <c r="U19" t="n">
+        <v>3.603598038258197e-18</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-2.624982417201998e-19</v>
       </c>
     </row>
     <row r="20">
@@ -3141,58 +3757,67 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-1.888440434176897</v>
+        <v>-2.374987233189456</v>
       </c>
       <c r="C20" t="n">
-        <v>-1.28566382924301</v>
+        <v>-1.267068303983673</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.007311257065743</v>
+        <v>-1.42594114123547</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1507429120969501</v>
+        <v>-0.3050834369932599</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.6260598185892906</v>
+        <v>0.2989871742263598</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.3537326145183517</v>
+        <v>0.3907149526701452</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.07633457164120434</v>
+        <v>-0.5636881338893732</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.06985638047757212</v>
+        <v>-0.3170985051069918</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3428272283278891</v>
+        <v>0.1894961154634598</v>
       </c>
       <c r="K20" t="n">
-        <v>0.129758643252488</v>
+        <v>0.01367145373698673</v>
       </c>
       <c r="L20" t="n">
-        <v>0.1502555980541071</v>
+        <v>0.0324653712578286</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0106387515922173</v>
+        <v>-0.03138714352366152</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.007799939678218976</v>
+        <v>-0.0059731184357991</v>
       </c>
       <c r="O20" t="n">
-        <v>0.01268941385363708</v>
+        <v>0.03886792803582714</v>
       </c>
       <c r="P20" t="n">
-        <v>0.01666866453731865</v>
+        <v>0.01684177615710613</v>
       </c>
       <c r="Q20" t="n">
-        <v>-0.006608152424999049</v>
+        <v>-0.006233525574854266</v>
       </c>
       <c r="R20" t="n">
-        <v>-7.133567673349404e-18</v>
+        <v>0.0150574070449434</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.013259426819103e-19</v>
+        <v>-0.0015199272944688</v>
+      </c>
+      <c r="T20" t="n">
+        <v>2.81824240215824e-17</v>
+      </c>
+      <c r="U20" t="n">
+        <v>1.303895416925733e-17</v>
+      </c>
+      <c r="V20" t="n">
+        <v>2.437352627293086e-19</v>
       </c>
     </row>
     <row r="21">
@@ -3202,58 +3827,67 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-2.151018865687908</v>
+        <v>-2.172601862781816</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.4988642226899411</v>
+        <v>-1.064803182012586</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.07258815228989327</v>
+        <v>-0.9322606488952443</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.2886674268942079</v>
+        <v>-0.3913377192202475</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3209824025903138</v>
+        <v>-0.9062106398054566</v>
       </c>
       <c r="G21" t="n">
-        <v>0.02472541931235114</v>
+        <v>-0.4053416908014891</v>
       </c>
       <c r="H21" t="n">
-        <v>0.2443792983783982</v>
+        <v>-0.0250156274274075</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1583901276388961</v>
+        <v>0.1441558906443202</v>
       </c>
       <c r="J21" t="n">
-        <v>0.06777751961747755</v>
+        <v>0.3854599481600171</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1012648098911471</v>
+        <v>0.1017538386260986</v>
       </c>
       <c r="L21" t="n">
-        <v>0.05912708757144384</v>
+        <v>0.1155280696411892</v>
       </c>
       <c r="M21" t="n">
-        <v>0.01482057103286565</v>
+        <v>0.1024544977939386</v>
       </c>
       <c r="N21" t="n">
-        <v>0.0162489895374485</v>
+        <v>0.02822413348342064</v>
       </c>
       <c r="O21" t="n">
-        <v>3.116106818556708e-05</v>
+        <v>-0.02323227915929593</v>
       </c>
       <c r="P21" t="n">
-        <v>-0.007762797537497854</v>
+        <v>0.03252100181429554</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.005619337405225027</v>
+        <v>-0.001845044932487522</v>
       </c>
       <c r="R21" t="n">
-        <v>-2.546261110579915e-17</v>
+        <v>-0.004972751441937703</v>
       </c>
       <c r="S21" t="n">
-        <v>-2.846772172050219e-20</v>
+        <v>0.0003688596019803611</v>
+      </c>
+      <c r="T21" t="n">
+        <v>7.208722565963927e-17</v>
+      </c>
+      <c r="U21" t="n">
+        <v>-1.909341095565369e-17</v>
+      </c>
+      <c r="V21" t="n">
+        <v>3.566431235673935e-20</v>
       </c>
     </row>
     <row r="22">
@@ -3263,58 +3897,67 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-2.075268270034464</v>
+        <v>-2.307580917193089</v>
       </c>
       <c r="C22" t="n">
-        <v>0.04815669840461035</v>
+        <v>0.1261745077657613</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.5575467248998303</v>
+        <v>-0.4504641975902029</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.0614661856459592</v>
+        <v>-0.4528440115091972</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1465792028800021</v>
+        <v>-0.2995615827220161</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4951902517974857</v>
+        <v>-0.002573360408214835</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2165891167583675</v>
+        <v>0.2691391546220059</v>
       </c>
       <c r="I22" t="n">
-        <v>0.02096850914800794</v>
+        <v>-0.2014026991472832</v>
       </c>
       <c r="J22" t="n">
-        <v>0.08882592621745247</v>
+        <v>0.1256803366916676</v>
       </c>
       <c r="K22" t="n">
-        <v>-0.07433725108836706</v>
+        <v>-0.04354453305293608</v>
       </c>
       <c r="L22" t="n">
-        <v>0.04491725710817637</v>
+        <v>0.03146898839659588</v>
       </c>
       <c r="M22" t="n">
-        <v>0.004382194350270866</v>
+        <v>0.06230102159847837</v>
       </c>
       <c r="N22" t="n">
-        <v>0.05935243378614505</v>
+        <v>0.02399856318764631</v>
       </c>
       <c r="O22" t="n">
-        <v>-0.003250227329878335</v>
+        <v>-0.002288285270990233</v>
       </c>
       <c r="P22" t="n">
-        <v>0.02367754633685587</v>
+        <v>-0.01142637598123738</v>
       </c>
       <c r="Q22" t="n">
-        <v>-0.006572213731882622</v>
+        <v>0.01288924329460606</v>
       </c>
       <c r="R22" t="n">
-        <v>-6.758028685895034e-19</v>
+        <v>0.0002744393339997582</v>
       </c>
       <c r="S22" t="n">
-        <v>4.071871348395613e-19</v>
+        <v>-0.00115203848393299</v>
+      </c>
+      <c r="T22" t="n">
+        <v>6.850237409595281e-17</v>
+      </c>
+      <c r="U22" t="n">
+        <v>4.17667535366583e-17</v>
+      </c>
+      <c r="V22" t="n">
+        <v>6.765332457489301e-19</v>
       </c>
     </row>
     <row r="23">
@@ -3324,58 +3967,67 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.6920766353228729</v>
+        <v>-2.316989591821458</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.1023951958760968</v>
+        <v>-0.7138607747081931</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1008114433108298</v>
+        <v>0.2519504833631355</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6978795101150544</v>
+        <v>0.007667664190161516</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.3288297790725573</v>
+        <v>0.1759085049577643</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1719697134081303</v>
+        <v>0.493894075243709</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.5515641227008</v>
+        <v>0.2240120645025345</v>
       </c>
       <c r="I23" t="n">
-        <v>0.006661777691369552</v>
+        <v>-0.1036643170215865</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.2792816035815391</v>
+        <v>0.05657076377812589</v>
       </c>
       <c r="K23" t="n">
-        <v>0.2278917109692917</v>
+        <v>0.1073140037583511</v>
       </c>
       <c r="L23" t="n">
-        <v>0.05503764413241971</v>
+        <v>0.06133813608921574</v>
       </c>
       <c r="M23" t="n">
-        <v>-0.01226804313695881</v>
+        <v>0.01010141129198599</v>
       </c>
       <c r="N23" t="n">
-        <v>0.05707599182516761</v>
+        <v>0.05383058029512587</v>
       </c>
       <c r="O23" t="n">
-        <v>-0.02408810311263115</v>
+        <v>0.0184559029251701</v>
       </c>
       <c r="P23" t="n">
-        <v>0.02181863970948184</v>
+        <v>0.009177525214005477</v>
       </c>
       <c r="Q23" t="n">
-        <v>-0.009634849795917428</v>
+        <v>-0.0001662164533579593</v>
       </c>
       <c r="R23" t="n">
-        <v>-2.691914956213542e-17</v>
+        <v>-0.006718311696227825</v>
       </c>
       <c r="S23" t="n">
-        <v>-2.373883638667052e-19</v>
+        <v>0.0003919453261245935</v>
+      </c>
+      <c r="T23" t="n">
+        <v>-1.099596604983853e-16</v>
+      </c>
+      <c r="U23" t="n">
+        <v>1.632113308166317e-17</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5.712246088968464e-19</v>
       </c>
     </row>
     <row r="24">
@@ -3385,58 +4037,67 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.589475945579051</v>
+        <v>-0.7833152592315394</v>
       </c>
       <c r="C24" t="n">
-        <v>2.09833772972532</v>
+        <v>0.1525506014914556</v>
       </c>
       <c r="D24" t="n">
-        <v>1.263664313004268</v>
+        <v>-0.09419141916321845</v>
       </c>
       <c r="E24" t="n">
-        <v>-1.251679922002106</v>
+        <v>0.5113139884817072</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.3862976701886664</v>
+        <v>-0.6046525653033281</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.6540960885318298</v>
+        <v>-0.2259253535067671</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.2323476460832037</v>
+        <v>-0.5595963210882108</v>
       </c>
       <c r="I24" t="n">
-        <v>0.02743614435302434</v>
+        <v>0.09247279422868739</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1484711336825026</v>
+        <v>-0.03628697862170079</v>
       </c>
       <c r="K24" t="n">
-        <v>-0.06236480892200093</v>
+        <v>-0.3726040442510769</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.001200674287883041</v>
+        <v>0.03204126350001824</v>
       </c>
       <c r="M24" t="n">
-        <v>-0.001020741715475788</v>
+        <v>0.05354757047284463</v>
       </c>
       <c r="N24" t="n">
-        <v>0.04281498440343133</v>
+        <v>0.08754133361382629</v>
       </c>
       <c r="O24" t="n">
-        <v>-0.03103257172660757</v>
+        <v>-0.01883701991806562</v>
       </c>
       <c r="P24" t="n">
-        <v>-0.004967109515933287</v>
+        <v>0.005047979750787487</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.005802222325037061</v>
+        <v>-0.005199971232374393</v>
       </c>
       <c r="R24" t="n">
-        <v>-2.576258879216532e-17</v>
+        <v>-0.008293345646563546</v>
       </c>
       <c r="S24" t="n">
-        <v>-3.874159173612116e-18</v>
+        <v>8.699140636682331e-05</v>
+      </c>
+      <c r="T24" t="n">
+        <v>-1.337190545471058e-17</v>
+      </c>
+      <c r="U24" t="n">
+        <v>5.553897429670056e-18</v>
+      </c>
+      <c r="V24" t="n">
+        <v>4.435703021173133e-19</v>
       </c>
     </row>
     <row r="25">
@@ -3446,58 +4107,67 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-2.051504884962058</v>
+        <v>3.059615023279903</v>
       </c>
       <c r="C25" t="n">
-        <v>0.468942013981481</v>
+        <v>2.789817623852149</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.7942807094054373</v>
+        <v>1.606594256377478</v>
       </c>
       <c r="E25" t="n">
-        <v>0.07119428355215227</v>
+        <v>-1.248518351411291</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.0867049975407274</v>
+        <v>0.08563633739933199</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1886628213347447</v>
+        <v>-0.6036496053533832</v>
       </c>
       <c r="H25" t="n">
-        <v>0.2566702219406772</v>
+        <v>-0.2436997699337939</v>
       </c>
       <c r="I25" t="n">
-        <v>0.03754941178236344</v>
+        <v>0.05908339923108625</v>
       </c>
       <c r="J25" t="n">
-        <v>0.02696648064898327</v>
+        <v>0.05348706089034171</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.1357450359558077</v>
+        <v>0.1526929427873679</v>
       </c>
       <c r="L25" t="n">
-        <v>0.0308156230905021</v>
+        <v>-0.001975270156026034</v>
       </c>
       <c r="M25" t="n">
-        <v>0.007801400621507075</v>
+        <v>5.819342704425552e-05</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.01179895192337467</v>
+        <v>0.04232334084374779</v>
       </c>
       <c r="O25" t="n">
-        <v>0.004921331427073626</v>
+        <v>-0.007514884710298321</v>
       </c>
       <c r="P25" t="n">
-        <v>0.009394897851817798</v>
+        <v>-0.02844290306147677</v>
       </c>
       <c r="Q25" t="n">
-        <v>-0.006809346380130813</v>
+        <v>0.0003174683142397593</v>
       </c>
       <c r="R25" t="n">
-        <v>5.484060317501741e-17</v>
+        <v>0.006035221863075439</v>
       </c>
       <c r="S25" t="n">
-        <v>1.749229402186149e-21</v>
+        <v>0.0004341698108682623</v>
+      </c>
+      <c r="T25" t="n">
+        <v>-1.998109798289772e-16</v>
+      </c>
+      <c r="U25" t="n">
+        <v>2.382967508207521e-17</v>
+      </c>
+      <c r="V25" t="n">
+        <v>5.460255736803854e-19</v>
       </c>
     </row>
     <row r="26">
@@ -3507,58 +4177,67 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.8304172298501795</v>
+        <v>-2.241491323387164</v>
       </c>
       <c r="C26" t="n">
-        <v>1.129109567550707</v>
+        <v>-0.5189842937758795</v>
       </c>
       <c r="D26" t="n">
-        <v>0.01005398239303134</v>
+        <v>0.713871951551296</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.335119161042685</v>
+        <v>-0.1340545477089212</v>
       </c>
       <c r="F26" t="n">
-        <v>0.5402432082518132</v>
+        <v>-0.2414237902549451</v>
       </c>
       <c r="G26" t="n">
-        <v>1.028985621266393</v>
+        <v>-0.2377645488004739</v>
       </c>
       <c r="H26" t="n">
-        <v>0.5253836118691168</v>
+        <v>0.2766187664715842</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.0572713752830917</v>
+        <v>-0.07237023885553787</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1169399772567543</v>
+        <v>-0.06155983091344797</v>
       </c>
       <c r="K26" t="n">
-        <v>0.03988951428027422</v>
+        <v>0.1209676875927014</v>
       </c>
       <c r="L26" t="n">
-        <v>0.06389085584966039</v>
+        <v>0.05193497900911134</v>
       </c>
       <c r="M26" t="n">
-        <v>-0.05161952489976897</v>
+        <v>-0.01823890443137998</v>
       </c>
       <c r="N26" t="n">
-        <v>-0.02176433731152434</v>
+        <v>-0.030237983435406</v>
       </c>
       <c r="O26" t="n">
-        <v>-0.04631029326925369</v>
+        <v>0.008258751370371856</v>
       </c>
       <c r="P26" t="n">
-        <v>0.002738139778784836</v>
+        <v>0.005561181643874139</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.007293940658989986</v>
+        <v>0.005846835776051437</v>
       </c>
       <c r="R26" t="n">
-        <v>-4.42271182767766e-17</v>
+        <v>-0.01084881700628109</v>
       </c>
       <c r="S26" t="n">
-        <v>1.927717117882199e-18</v>
+        <v>-0.0004807476921439658</v>
+      </c>
+      <c r="T26" t="n">
+        <v>2.802918301496982e-17</v>
+      </c>
+      <c r="U26" t="n">
+        <v>-4.110732537458812e-18</v>
+      </c>
+      <c r="V26" t="n">
+        <v>2.747295576234462e-19</v>
       </c>
     </row>
     <row r="27">
@@ -3568,58 +4247,67 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8.361279828529446</v>
+        <v>-0.883686275451408</v>
       </c>
       <c r="C27" t="n">
-        <v>-1.422545697026402</v>
+        <v>-0.1352948756967656</v>
       </c>
       <c r="D27" t="n">
-        <v>0.5968836794854684</v>
+        <v>1.148645721991379</v>
       </c>
       <c r="E27" t="n">
-        <v>1.232750979143935</v>
+        <v>0.1872314294287692</v>
       </c>
       <c r="F27" t="n">
-        <v>-3.124441298239125</v>
+        <v>0.881415489923901</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5121895434002083</v>
+        <v>1.138828492794129</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1766176504222506</v>
+        <v>0.5498646484987</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.03222894038872992</v>
+        <v>-0.08580743677480003</v>
       </c>
       <c r="J27" t="n">
-        <v>-0.02750154976802619</v>
+        <v>0.1360176036123154</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.05832328221831883</v>
+        <v>0.03756361680266544</v>
       </c>
       <c r="L27" t="n">
-        <v>-0.006726024464907595</v>
+        <v>0.06596938200807666</v>
       </c>
       <c r="M27" t="n">
-        <v>0.01000694911742162</v>
+        <v>-0.01885602083589209</v>
       </c>
       <c r="N27" t="n">
-        <v>0.002347730252918863</v>
+        <v>0.01373310460392501</v>
       </c>
       <c r="O27" t="n">
-        <v>-0.002312726790429185</v>
+        <v>-0.06440820469116726</v>
       </c>
       <c r="P27" t="n">
-        <v>-0.007416303764439141</v>
+        <v>-0.01472789361722568</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.001820250971962841</v>
+        <v>0.001191187103768753</v>
       </c>
       <c r="R27" t="n">
-        <v>-1.858339463974031e-17</v>
+        <v>0.007014555424978288</v>
       </c>
       <c r="S27" t="n">
-        <v>-1.527123495979347e-19</v>
+        <v>-0.0007158979236996339</v>
+      </c>
+      <c r="T27" t="n">
+        <v>1.972848357942437e-17</v>
+      </c>
+      <c r="U27" t="n">
+        <v>5.648573642736877e-18</v>
+      </c>
+      <c r="V27" t="n">
+        <v>-1.512885979934394e-19</v>
       </c>
     </row>
     <row r="28">
@@ -3629,58 +4317,137 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.1092670670872819</v>
+        <v>9.438948388141375</v>
       </c>
       <c r="C28" t="n">
-        <v>-2.285149125796217</v>
+        <v>0.6975185435360449</v>
       </c>
       <c r="D28" t="n">
-        <v>1.713003788963565</v>
+        <v>-1.528177063448392</v>
       </c>
       <c r="E28" t="n">
-        <v>-1.582609562797971</v>
+        <v>0.2288485649485934</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4749191412927455</v>
+        <v>-3.337761174268459</v>
       </c>
       <c r="G28" t="n">
-        <v>0.03112864819013988</v>
+        <v>0.8856147550470903</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.03681323419959542</v>
+        <v>0.1528722366950815</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.3092160975177564</v>
+        <v>0.01431163767377158</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.1353276722643036</v>
+        <v>-0.08303017937144502</v>
       </c>
       <c r="K28" t="n">
-        <v>0.02282465233687208</v>
+        <v>0.04115991718094093</v>
       </c>
       <c r="L28" t="n">
-        <v>-0.04037312255667153</v>
+        <v>0.002424760109625391</v>
       </c>
       <c r="M28" t="n">
-        <v>0.0519752181675476</v>
+        <v>-0.006373853259016821</v>
       </c>
       <c r="N28" t="n">
-        <v>-0.008580970544088283</v>
+        <v>-0.008720614516611595</v>
       </c>
       <c r="O28" t="n">
-        <v>-0.03105852388621247</v>
+        <v>0.007349273146363586</v>
       </c>
       <c r="P28" t="n">
-        <v>0.01228452733607002</v>
+        <v>-0.01042471635123478</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.01117389787848671</v>
+        <v>-0.0002691848652467734</v>
       </c>
       <c r="R28" t="n">
-        <v>-3.422874941481027e-18</v>
+        <v>0.001709580408583219</v>
       </c>
       <c r="S28" t="n">
-        <v>2.103266408908863e-19</v>
+        <v>-0.0001550993296763282</v>
+      </c>
+      <c r="T28" t="n">
+        <v>3.111002832101683e-17</v>
+      </c>
+      <c r="U28" t="n">
+        <v>8.470792380746439e-18</v>
+      </c>
+      <c r="V28" t="n">
+        <v>2.616744081000344e-19</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nisin</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.1720814411612505</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.209351506508505</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-2.720292531577199</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-0.9859718360535245</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.163339009739059</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.2315467122260385</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.06039164273590276</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.4271100987988509</v>
+      </c>
+      <c r="J29" t="n">
+        <v>-0.0968504247867415</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-0.09263542755140945</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-0.050891560863426</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.02848278401469516</v>
+      </c>
+      <c r="N29" t="n">
+        <v>-0.01805014229535572</v>
+      </c>
+      <c r="O29" t="n">
+        <v>-0.02542871348794228</v>
+      </c>
+      <c r="P29" t="n">
+        <v>-0.01535536138089951</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.01722705432924101</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.003747426807108236</v>
+      </c>
+      <c r="S29" t="n">
+        <v>-0.002058826160789251</v>
+      </c>
+      <c r="T29" t="n">
+        <v>8.955311737360115e-18</v>
+      </c>
+      <c r="U29" t="n">
+        <v>-2.576731326684943e-17</v>
+      </c>
+      <c r="V29" t="n">
+        <v>3.832400271889714e-19</v>
       </c>
     </row>
   </sheetData>
@@ -3694,7 +4461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3770,42 +4537,57 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>aliphatic_ring_count</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>saturated_ring_count</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>fraction_csp3</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>heteroatom_count</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>formal_charge</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>atom_count</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>amide_bond_count</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>defined_atom_stereocenter_count</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>defined_bond_stereocenter_count</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>molar_refractivity</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>labute_surface_area</t>
         </is>
       </c>
     </row>
@@ -3858,17 +4640,20 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="n">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="n">
         <v>6</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>0</v>
       </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Glatiramer acetate</t>
+          <t>Granulocyte-Colony Stimulating Factor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3883,26 +4668,28 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>623.7</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>727.8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-5.3</v>
+      </c>
       <c r="G3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" t="n">
         <v>13</v>
-      </c>
-      <c r="H3" t="n">
-        <v>18</v>
       </c>
       <c r="I3" t="n">
         <v>12</v>
       </c>
       <c r="J3" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="K3" t="n">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="L3" t="n">
-        <v>519</v>
+        <v>1170</v>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -3912,68 +4699,15 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="n">
-        <v>4</v>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
+        <v>7</v>
+      </c>
+      <c r="W3" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Granulocyte-Colony Stimulating Factor</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Manual backup</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>727.8</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="G4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H4" t="n">
-        <v>13</v>
-      </c>
-      <c r="I4" t="n">
-        <v>12</v>
-      </c>
-      <c r="J4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" t="n">
-        <v>359</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1170</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>